<commit_message>
GQ-Kategorie: 32 Gruppenqualifikanten +3 Pkt je Treffer
- Neue Scoring-Kategorie "GQ": welche 32 Teams kommen aus der Gruppenphase?
  Wird automatisch aus den 72 Spieltipps berechnet (kein extra Tipp nötig)
- calc_qualifiers_from_predictions(): Port der tippzettel.js-Logik nach Python
- S16 (16 Weiterkommer aus dem S16) von +3 auf +5 Pkt erhöht
- GQ-Tab in Detailauswertung: ✓/✗ Matrix für alle 32 Qualifikanten
- Legende aktualisiert; Ranking-Tabelle + Excel-Rangliste mit GQ-Spalte
- tippzettel.html: S16 pts 3→5, q-box Hinweis "+3 Pkt/Qualifikant"
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -532,12 +532,13 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -563,35 +564,40 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t>Gr.-Qualifikation</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t>Sechzehntelfinale</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Achtelfinale</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Viertelfinale</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Halbfinale</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Platz 3</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Finale</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Weltmeister</t>
         </is>
@@ -633,6 +639,9 @@
       <c r="K2" s="4" t="n">
         <v>0</v>
       </c>
+      <c r="L2" s="4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="5" t="n">
@@ -670,6 +679,9 @@
       <c r="K3" s="7" t="n">
         <v>0</v>
       </c>
+      <c r="L3" s="7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="n">
@@ -705,6 +717,9 @@
         <v>0</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update: Neue Test-Tipps + Rangliste aktualisiert
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -524,7 +524,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -532,13 +532,12 @@
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -569,35 +568,30 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Sechzehntelfinale</t>
+          <t>Achtelfinale</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Achtelfinale</t>
+          <t>Viertelfinale</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Viertelfinale</t>
+          <t>Halbfinale</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Halbfinale</t>
+          <t>Platz 3</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Platz 3</t>
+          <t>Finale</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>Finale</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Weltmeister</t>
         </is>
@@ -609,7 +603,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Test 2 Rathaus</t>
+          <t>Timo Test1</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -637,9 +631,6 @@
         <v>0</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -649,7 +640,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Timo Mayer</t>
+          <t>Timo Test2</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -677,9 +668,6 @@
         <v>0</v>
       </c>
       <c r="K3" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="L3" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -689,7 +677,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Timo Test</t>
+          <t>Timo Test2</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
@@ -717,9 +705,6 @@
         <v>0</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -757,17 +742,17 @@
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Test 2 Rathaus</t>
+          <t>Timo Test1</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>Timo Mayer</t>
+          <t>Timo Test2</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Timo Test</t>
+          <t>Timo Test2</t>
         </is>
       </c>
     </row>
@@ -791,17 +776,17 @@
       </c>
       <c r="C3" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:5</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>5:4</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>5:4</t>
         </is>
       </c>
     </row>
@@ -818,17 +803,17 @@
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>1:5</t>
         </is>
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>4:5</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>4:2</t>
         </is>
       </c>
     </row>
@@ -845,17 +830,17 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="E5" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -872,17 +857,17 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="D6" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E6" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -899,17 +884,17 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>7:3</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>4:25</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:4</t>
         </is>
       </c>
     </row>
@@ -926,17 +911,17 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>2:3</t>
+          <t>7:8</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>2:3</t>
+          <t>4:5</t>
         </is>
       </c>
     </row>
@@ -960,17 +945,17 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:5</t>
         </is>
       </c>
     </row>
@@ -987,17 +972,17 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D11" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>4:5</t>
         </is>
       </c>
     </row>
@@ -1014,7 +999,7 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -1024,7 +1009,7 @@
       </c>
       <c r="E12" s="15" t="inlineStr">
         <is>
-          <t>3:2</t>
+          <t>1:2</t>
         </is>
       </c>
     </row>
@@ -1041,17 +1026,17 @@
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1068,7 +1053,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:18</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
@@ -1078,7 +1063,7 @@
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>3:3</t>
+          <t>1:2</t>
         </is>
       </c>
     </row>
@@ -1095,17 +1080,17 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>6:8</t>
         </is>
       </c>
       <c r="D15" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E15" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:2</t>
         </is>
       </c>
     </row>
@@ -1129,17 +1114,17 @@
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D17" s="15" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E17" s="15" t="inlineStr">
         <is>
-          <t>3:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1156,17 +1141,17 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>0:6</t>
+          <t>8:8</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>1:5</t>
         </is>
       </c>
     </row>
@@ -1183,17 +1168,17 @@
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>4:4</t>
         </is>
       </c>
       <c r="D19" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="E19" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:52</t>
         </is>
       </c>
     </row>
@@ -1210,17 +1195,17 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>5:2</t>
+          <t>1:2</t>
         </is>
       </c>
     </row>
@@ -1237,17 +1222,17 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -1264,17 +1249,17 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>8:84</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1298,17 +1283,17 @@
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>8:1</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>3:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1325,12 +1310,12 @@
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
@@ -1352,17 +1337,17 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:5</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1379,7 +1364,7 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>5:8</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
@@ -1389,7 +1374,7 @@
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>5:5</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1406,17 +1391,17 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>5:48</t>
         </is>
       </c>
       <c r="D28" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="E28" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1433,17 +1418,17 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:58</t>
         </is>
       </c>
       <c r="D29" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1467,17 +1452,17 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>6:0</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D31" s="15" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1494,12 +1479,12 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>2:3</t>
+          <t>8:5</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
@@ -1521,12 +1506,12 @@
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:48</t>
         </is>
       </c>
       <c r="D33" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E33" s="15" t="inlineStr">
@@ -1548,17 +1533,17 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>5:1</t>
+          <t>5:8</t>
         </is>
       </c>
       <c r="D34" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="E34" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1575,17 +1560,17 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>0:6</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1602,7 +1587,7 @@
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>1:8</t>
         </is>
       </c>
       <c r="D36" s="15" t="inlineStr">
@@ -1612,7 +1597,7 @@
       </c>
       <c r="E36" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1636,17 +1621,17 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>5:8</t>
         </is>
       </c>
       <c r="D38" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E38" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1663,17 +1648,17 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>1:8</t>
         </is>
       </c>
       <c r="D39" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="E39" s="15" t="inlineStr">
         <is>
-          <t>0:02</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1690,17 +1675,17 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D40" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E40" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1717,7 +1702,7 @@
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>4:5</t>
         </is>
       </c>
       <c r="D41" s="15" t="inlineStr">
@@ -1727,7 +1712,7 @@
       </c>
       <c r="E41" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1744,17 +1729,17 @@
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D42" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="E42" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1771,17 +1756,17 @@
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>8:5</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1805,17 +1790,17 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1832,17 +1817,17 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:21</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1859,17 +1844,17 @@
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D47" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E47" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1886,17 +1871,17 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>8:5</t>
         </is>
       </c>
       <c r="D48" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E48" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1913,17 +1898,17 @@
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>5:4</t>
         </is>
       </c>
       <c r="D49" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E49" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1940,17 +1925,17 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>8:5</t>
         </is>
       </c>
       <c r="D50" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="E50" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1974,17 +1959,17 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>5:0</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D52" s="15" t="inlineStr">
         <is>
-          <t>5:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E52" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2001,17 +1986,17 @@
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>8:5</t>
         </is>
       </c>
       <c r="D53" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E53" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2028,17 +2013,17 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:5</t>
         </is>
       </c>
       <c r="D54" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E54" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2055,17 +2040,17 @@
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D55" s="15" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E55" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2082,17 +2067,17 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:8</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2109,17 +2094,17 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D57" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>1:21</t>
         </is>
       </c>
       <c r="E57" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2143,17 +2128,17 @@
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="D59" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E59" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2170,17 +2155,17 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>0:5</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="D60" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E60" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2197,17 +2182,17 @@
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D61" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:21</t>
         </is>
       </c>
       <c r="E61" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2224,17 +2209,17 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>8:2</t>
         </is>
       </c>
       <c r="D62" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E62" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2251,17 +2236,17 @@
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>4:28</t>
         </is>
       </c>
       <c r="D63" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E63" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2278,7 +2263,7 @@
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>8:4</t>
         </is>
       </c>
       <c r="D64" s="15" t="inlineStr">
@@ -2288,7 +2273,7 @@
       </c>
       <c r="E64" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2312,17 +2297,17 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D66" s="15" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E66" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2339,17 +2324,17 @@
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:8</t>
         </is>
       </c>
       <c r="D67" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E67" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2366,17 +2351,17 @@
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:4</t>
         </is>
       </c>
       <c r="D68" s="15" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E68" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2393,17 +2378,17 @@
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2420,17 +2405,17 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>1:3</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E70" s="15" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>1:2</t>
         </is>
       </c>
     </row>
@@ -2447,17 +2432,17 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>0:5</t>
+          <t>1:5</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E71" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2481,17 +2466,17 @@
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>5:1</t>
         </is>
       </c>
       <c r="D73" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E73" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2508,12 +2493,12 @@
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D74" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E74" s="15" t="inlineStr">
@@ -2535,17 +2520,17 @@
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D75" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>1:21</t>
         </is>
       </c>
       <c r="E75" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2562,17 +2547,17 @@
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>5:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D76" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E76" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2589,17 +2574,17 @@
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="D77" s="15" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="D77" s="15" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
       <c r="E77" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2616,17 +2601,17 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D78" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E78" s="15" t="inlineStr">
         <is>
-          <t>1:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2650,17 +2635,17 @@
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D80" s="15" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E80" s="15" t="inlineStr">
         <is>
-          <t>1:2</t>
+          <t>2:12</t>
         </is>
       </c>
     </row>
@@ -2677,17 +2662,17 @@
       </c>
       <c r="C81" s="15" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D81" s="15" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="E81" s="15" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2709,12 +2694,12 @@
       </c>
       <c r="D82" s="15" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E82" s="15" t="inlineStr">
         <is>
-          <t>0:5</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2731,17 +2716,17 @@
       </c>
       <c r="C83" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="D83" s="15" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E83" s="15" t="inlineStr">
         <is>
-          <t>4:4</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2758,17 +2743,17 @@
       </c>
       <c r="C84" s="15" t="inlineStr">
         <is>
-          <t>0:1</t>
+          <t>2:21</t>
         </is>
       </c>
       <c r="D84" s="15" t="inlineStr">
         <is>
-          <t>0:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="E84" s="15" t="inlineStr">
         <is>
-          <t>4:5</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2770,7 @@
       </c>
       <c r="C85" s="15" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>1:2</t>
         </is>
       </c>
       <c r="D85" s="15" t="inlineStr">
@@ -2795,7 +2780,7 @@
       </c>
       <c r="E85" s="15" t="inlineStr">
         <is>
-          <t>4:5</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2824,7 +2809,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2847,24 +2832,24 @@
       </c>
       <c r="C1" s="11" t="inlineStr">
         <is>
-          <t>Test 2 Rathaus</t>
+          <t>Timo Test1</t>
         </is>
       </c>
       <c r="D1" s="11" t="inlineStr">
         <is>
-          <t>Timo Mayer</t>
+          <t>Timo Test2</t>
         </is>
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Timo Test</t>
+          <t>Timo Test2</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>── Sechzehntelfinale (je 5 Pkt.) ──</t>
+          <t>── Achtelfinale-Teilnehmer (16) (je 5 Pkt.) ──</t>
         </is>
       </c>
     </row>
@@ -2886,7 +2871,7 @@
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>Mexiko</t>
+          <t>Kanada</t>
         </is>
       </c>
       <c r="E3" s="15" t="inlineStr">
@@ -2913,12 +2898,12 @@
       </c>
       <c r="D4" s="15" t="inlineStr">
         <is>
-          <t>Brasilien</t>
+          <t>Marokko</t>
         </is>
       </c>
       <c r="E4" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
@@ -2935,7 +2920,7 @@
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Elfenbeinküste</t>
         </is>
       </c>
       <c r="D5" s="15" t="inlineStr">
@@ -2962,17 +2947,17 @@
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="D6" s="15" t="inlineStr">
+        <is>
+          <t>Schweden</t>
+        </is>
+      </c>
+      <c r="E6" s="15" t="inlineStr">
+        <is>
           <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="D6" s="15" t="inlineStr">
-        <is>
-          <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="E6" s="15" t="inlineStr">
-        <is>
-          <t>Brasilien</t>
         </is>
       </c>
     </row>
@@ -2989,12 +2974,12 @@
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Norwegen</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="D7" s="15" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="E7" s="15" t="inlineStr">
@@ -3016,17 +3001,17 @@
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Iran</t>
         </is>
       </c>
       <c r="D8" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Schottland</t>
         </is>
       </c>
       <c r="E8" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Australien</t>
         </is>
       </c>
     </row>
@@ -3043,17 +3028,17 @@
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="D9" s="15" t="inlineStr">
+        <is>
           <t>Mexiko</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
-        <is>
-          <t>Tschechien</t>
-        </is>
-      </c>
       <c r="E9" s="15" t="inlineStr">
         <is>
-          <t>Tschechien</t>
+          <t>Mexiko</t>
         </is>
       </c>
     </row>
@@ -3070,17 +3055,17 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Usbekistan</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="E10" s="15" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Kroatien</t>
         </is>
       </c>
     </row>
@@ -3097,17 +3082,17 @@
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="D11" s="15" t="inlineStr">
+        <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
-        <is>
-          <t>Ägypten</t>
-        </is>
-      </c>
       <c r="E11" s="15" t="inlineStr">
         <is>
-          <t>Ägypten</t>
+          <t>Belgien</t>
         </is>
       </c>
     </row>
@@ -3124,17 +3109,17 @@
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
+          <t>Australien</t>
+        </is>
+      </c>
+      <c r="D12" s="15" t="inlineStr">
+        <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="E12" s="15" t="inlineStr">
+        <is>
           <t>Türkei</t>
-        </is>
-      </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>Türkei</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
-        <is>
-          <t>Portugal</t>
         </is>
       </c>
     </row>
@@ -3156,12 +3141,12 @@
       </c>
       <c r="D13" s="15" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>Argentinien</t>
         </is>
       </c>
       <c r="E13" s="15" t="inlineStr">
         <is>
-          <t>Österreich</t>
+          <t>Jordanien</t>
         </is>
       </c>
     </row>
@@ -3178,17 +3163,17 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Kroatien</t>
+          <t>Kolumbien</t>
         </is>
       </c>
       <c r="D14" s="15" t="inlineStr">
         <is>
-          <t>Kolumbien</t>
+          <t>England</t>
         </is>
       </c>
       <c r="E14" s="15" t="inlineStr">
         <is>
-          <t>Kroatien</t>
+          <t>Portugal</t>
         </is>
       </c>
     </row>
@@ -3205,17 +3190,17 @@
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>Ägypten</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
+        <is>
           <t>Bosnien-Herzegowina</t>
-        </is>
-      </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>Schweiz</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
-        <is>
-          <t>Schweiz</t>
         </is>
       </c>
     </row>
@@ -3232,17 +3217,17 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D16" s="15" t="inlineStr">
         <is>
-          <t>Belgien</t>
+          <t>Türkei</t>
         </is>
       </c>
       <c r="E16" s="15" t="inlineStr">
         <is>
-          <t>Belgien</t>
+          <t>USA</t>
         </is>
       </c>
     </row>
@@ -3259,17 +3244,17 @@
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
+          <t>Jordanien</t>
+        </is>
+      </c>
+      <c r="D17" s="15" t="inlineStr">
+        <is>
+          <t>Algerien</t>
+        </is>
+      </c>
+      <c r="E17" s="15" t="inlineStr">
+        <is>
           <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="D17" s="15" t="inlineStr">
-        <is>
-          <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="E17" s="15" t="inlineStr">
-        <is>
-          <t>Spanien</t>
         </is>
       </c>
     </row>
@@ -3286,24 +3271,24 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Irak</t>
         </is>
       </c>
       <c r="D18" s="15" t="inlineStr">
         <is>
-          <t>Portugal</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>── Achtelfinale (je 10 Pkt.) ──</t>
+          <t>── Viertelfinale-Teilnehmer (8) (je 10 Pkt.) ──</t>
         </is>
       </c>
     </row>
@@ -3325,12 +3310,12 @@
       </c>
       <c r="D20" s="15" t="inlineStr">
         <is>
-          <t>Brasilien</t>
+          <t>Marokko</t>
         </is>
       </c>
       <c r="E20" s="15" t="inlineStr">
         <is>
-          <t>Japan</t>
+          <t>Marokko</t>
         </is>
       </c>
     </row>
@@ -3347,17 +3332,17 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+      <c r="D21" s="15" t="inlineStr">
+        <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Niederlande</t>
         </is>
       </c>
     </row>
@@ -3374,17 +3359,17 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Norwegen</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Schottland</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Australien</t>
         </is>
       </c>
     </row>
@@ -3401,17 +3386,17 @@
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Mexiko</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>Tschechien</t>
+          <t>Kroatien</t>
         </is>
       </c>
     </row>
@@ -3428,17 +3413,17 @@
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="D24" s="15" t="inlineStr">
+        <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>Ägypten</t>
-        </is>
-      </c>
       <c r="E24" s="15" t="inlineStr">
         <is>
-          <t>Ägypten</t>
+          <t>Türkei</t>
         </is>
       </c>
     </row>
@@ -3460,12 +3445,12 @@
       </c>
       <c r="D25" s="15" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>England</t>
         </is>
       </c>
       <c r="E25" s="15" t="inlineStr">
         <is>
-          <t>Kroatien</t>
+          <t>Portugal</t>
         </is>
       </c>
     </row>
@@ -3482,17 +3467,17 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Bosnien-Herzegowina</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D26" s="15" t="inlineStr">
         <is>
-          <t>Belgien</t>
+          <t>Ägypten</t>
         </is>
       </c>
       <c r="E26" s="15" t="inlineStr">
         <is>
-          <t>Belgien</t>
+          <t>USA</t>
         </is>
       </c>
     </row>
@@ -3509,24 +3494,24 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Argentinien</t>
+          <t>Irak</t>
         </is>
       </c>
       <c r="D27" s="15" t="inlineStr">
         <is>
-          <t>Argentinien</t>
+          <t>Algerien</t>
         </is>
       </c>
       <c r="E27" s="15" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="12" t="inlineStr">
         <is>
-          <t>── Viertelfinale (je 15 Pkt.) ──</t>
+          <t>── Halbfinale-Teilnehmer (4) (je 15 Pkt.) ──</t>
         </is>
       </c>
     </row>
@@ -3543,17 +3528,17 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
       <c r="E29" s="15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Niederlande</t>
         </is>
       </c>
     </row>
@@ -3570,17 +3555,17 @@
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>England</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="D30" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Schottland</t>
         </is>
       </c>
       <c r="E30" s="15" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Australien</t>
         </is>
       </c>
     </row>
@@ -3597,17 +3582,17 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
-        <is>
-          <t>Spanien</t>
-        </is>
-      </c>
       <c r="E31" s="15" t="inlineStr">
         <is>
-          <t>Kroatien</t>
+          <t>Türkei</t>
         </is>
       </c>
     </row>
@@ -3624,24 +3609,24 @@
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Argentinien</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D32" s="15" t="inlineStr">
         <is>
-          <t>Argentinien</t>
+          <t>Ägypten</t>
         </is>
       </c>
       <c r="E32" s="15" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>── Halbfinale (je 20 Pkt.) ──</t>
+          <t>── Finale (je 20 Pkt.) ──</t>
         </is>
       </c>
     </row>
@@ -3658,17 +3643,17 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
+          <t>Curaçao</t>
+        </is>
+      </c>
+      <c r="D34" s="15" t="inlineStr">
+        <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
       <c r="E34" s="15" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Niederlande</t>
         </is>
       </c>
     </row>
@@ -3685,24 +3670,24 @@
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Argentinien</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="D35" s="15" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>Ägypten</t>
         </is>
       </c>
       <c r="E35" s="15" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>── Finale (beide Finalisten) (je 25 Pkt.) ──</t>
+          <t>── Weltmeister (je 25 Pkt.) ──</t>
         </is>
       </c>
     </row>
@@ -3719,84 +3704,22 @@
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
       <c r="E37" s="15" t="inlineStr">
         <is>
-          <t>DR Kongo</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Weiterkommer 2</t>
-        </is>
-      </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C38" s="15" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" s="12" t="inlineStr">
-        <is>
-          <t>── Weltmeister (je 30 Pkt.) ──</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  Weiterkommer 1</t>
-        </is>
-      </c>
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
-        <is>
-          <t>DR Kongo</t>
+          <t>Curaçao</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
-    <mergeCell ref="A39:E39"/>
+  <mergeCells count="5">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A33:E33"/>

</xml_diff>

<commit_message>
Update: Tipps angepasst + Rangliste aktualisiert
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -677,7 +677,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Timo Test2</t>
+          <t>Timo Test3</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
@@ -752,7 +752,7 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Timo Test2</t>
+          <t>Timo Test3</t>
         </is>
       </c>
     </row>
@@ -2842,7 +2842,7 @@
       </c>
       <c r="E1" s="11" t="inlineStr">
         <is>
-          <t>Timo Test2</t>
+          <t>Timo Test3</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Neuer Tipp: italien hinzugefügt; Rangliste aktualisiert
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -118,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -145,6 +145,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -524,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -603,7 +609,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Timo Test1</t>
+          <t>italien</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -640,7 +646,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>Timo Test2</t>
+          <t>Timo Test1</t>
         </is>
       </c>
       <c r="C3" s="5" t="n">
@@ -677,7 +683,7 @@
       </c>
       <c r="B4" s="9" t="inlineStr">
         <is>
-          <t>Timo Test3</t>
+          <t>Timo Test2</t>
         </is>
       </c>
       <c r="C4" s="8" t="n">
@@ -705,6 +711,43 @@
         <v>0</v>
       </c>
       <c r="K4" s="4" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="10" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Timo Test3</t>
+        </is>
+      </c>
+      <c r="C5" s="10" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K5" s="7" t="n">
         <v>0</v>
       </c>
     </row>
@@ -719,7 +762,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:F85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -727,2058 +770,2424 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>Spiel</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Ergebnis</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>italien</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Timo Test1</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Timo Test2</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Timo Test3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>── Gruppe A ──</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Mexiko vs Südafrika (11.06.)</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>1:5</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>5:4</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>5:4</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Südkorea vs Tschechien (12.06.)</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>1:5</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>Tschechien vs Südafrika (18.06.)</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t>Mexiko vs Südkorea (19.06.)</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t>Tschechien vs Mexiko (25.06.)</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>7:3</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>4:25</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>2:4</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t>Südafrika vs Südkorea (25.06.)</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>7:8</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="14" t="inlineStr">
         <is>
           <t>── Gruppe B ──</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t>Kanada vs Bosnien-Herzegowina (12.06.)</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t>Katar vs Schweiz (13.06.)</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>Schweiz vs Bosnien-Herzegowina (18.06.)</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t>Kanada vs Katar (19.06.)</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t>Schweiz vs Kanada (24.06.)</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>1:18</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>Bosnien-Herzegowina vs Katar (24.06.)</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="D15" s="17" t="inlineStr">
         <is>
           <t>6:8</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E15" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>── Gruppe C ──</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t>Brasilien vs Marokko (14.06.)</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t>Haiti vs Schottland (14.06.)</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>8:8</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>1:5</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="15" t="inlineStr">
         <is>
           <t>Schottland vs Marokko (20.06.)</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="B19" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="inlineStr">
         <is>
           <t>4:4</t>
         </is>
       </c>
-      <c r="D19" s="15" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="E19" s="15" t="inlineStr">
+      <c r="F19" s="17" t="inlineStr">
         <is>
           <t>1:52</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t>Brasilien vs Haiti (20.06.)</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t>Schottland vs Brasilien (25.06.)</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t>Marokko vs Haiti (25.06.)</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>8:84</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>── Gruppe D ──</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t>USA vs Paraguay (13.06.)</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>8:1</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>Australien vs Türkei (14.06.)</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t>USA vs Australien (19.06.)</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F26" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>Türkei vs Paraguay (20.06.)</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>5:8</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F27" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="15" t="inlineStr">
         <is>
           <t>Türkei vs USA (26.06.)</t>
         </is>
       </c>
-      <c r="B28" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="B28" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C28" s="17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
         <is>
           <t>5:48</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
+      <c r="E28" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="E28" s="15" t="inlineStr">
+      <c r="F28" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t>Paraguay vs Australien (26.06.)</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>4:58</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F29" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>── Gruppe E ──</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t>Deutschland vs Curaçao (14.06.)</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t>Elfenbeinküste vs Ecuador (15.06.)</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>3:5</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>8:5</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="F32" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="13" t="inlineStr">
+      <c r="A33" s="15" t="inlineStr">
         <is>
           <t>Deutschland vs Elfenbeinküste (20.06.)</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C33" s="15" t="inlineStr">
+      <c r="B33" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C33" s="17" t="inlineStr">
+        <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="D33" s="17" t="inlineStr">
         <is>
           <t>4:48</t>
         </is>
       </c>
-      <c r="D33" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E33" s="15" t="inlineStr">
+      <c r="E33" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t>Ecuador vs Curaçao (21.06.)</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>5:8</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="F34" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t>Curaçao vs Elfenbeinküste (25.06.)</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="F35" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="13" t="inlineStr">
+      <c r="A36" s="15" t="inlineStr">
         <is>
           <t>Ecuador vs Deutschland (25.06.)</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
+      <c r="B36" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C36" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
         <is>
           <t>1:8</t>
         </is>
       </c>
-      <c r="D36" s="15" t="inlineStr">
+      <c r="E36" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E36" s="15" t="inlineStr">
+      <c r="F36" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="12" t="inlineStr">
+      <c r="A37" s="14" t="inlineStr">
         <is>
           <t>── Gruppe F ──</t>
         </is>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="13" t="inlineStr">
+      <c r="A38" s="15" t="inlineStr">
         <is>
           <t>Niederlande vs Japan (14.06.)</t>
         </is>
       </c>
-      <c r="B38" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C38" s="15" t="inlineStr">
+      <c r="B38" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C38" s="17" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
         <is>
           <t>5:8</t>
         </is>
       </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E38" s="15" t="inlineStr">
+      <c r="E38" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F38" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="13" t="inlineStr">
+      <c r="A39" s="15" t="inlineStr">
         <is>
           <t>Schweden vs Tunesien (15.06.)</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C39" s="15" t="inlineStr">
+      <c r="B39" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C39" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
         <is>
           <t>1:8</t>
         </is>
       </c>
-      <c r="D39" s="15" t="inlineStr">
+      <c r="E39" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="E39" s="15" t="inlineStr">
+      <c r="F39" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="40">
-      <c r="A40" s="13" t="inlineStr">
+      <c r="A40" s="15" t="inlineStr">
         <is>
           <t>Niederlande vs Schweden (20.06.)</t>
         </is>
       </c>
-      <c r="B40" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
+      <c r="B40" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C40" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D40" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D40" s="15" t="inlineStr">
+      <c r="E40" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E40" s="15" t="inlineStr">
+      <c r="F40" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="13" t="inlineStr">
+      <c r="A41" s="15" t="inlineStr">
         <is>
           <t>Tunesien vs Japan (21.06.)</t>
         </is>
       </c>
-      <c r="B41" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C41" s="15" t="inlineStr">
+      <c r="B41" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C41" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
-      <c r="D41" s="15" t="inlineStr">
+      <c r="E41" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E41" s="15" t="inlineStr">
+      <c r="F41" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="13" t="inlineStr">
+      <c r="A42" s="15" t="inlineStr">
         <is>
           <t>Japan vs Schweden (26.06.)</t>
         </is>
       </c>
-      <c r="B42" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
+      <c r="B42" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C42" s="17" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="D42" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D42" s="15" t="inlineStr">
+      <c r="E42" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="E42" s="15" t="inlineStr">
+      <c r="F42" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="43">
-      <c r="A43" s="13" t="inlineStr">
+      <c r="A43" s="15" t="inlineStr">
         <is>
           <t>Tunesien vs Niederlande (26.06.)</t>
         </is>
       </c>
-      <c r="B43" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
+      <c r="B43" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C43" s="17" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="D43" s="17" t="inlineStr">
         <is>
           <t>8:5</t>
         </is>
       </c>
-      <c r="D43" s="15" t="inlineStr">
+      <c r="E43" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E43" s="15" t="inlineStr">
+      <c r="F43" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="12" t="inlineStr">
+      <c r="A44" s="14" t="inlineStr">
         <is>
           <t>── Gruppe G ──</t>
         </is>
       </c>
     </row>
     <row r="45">
-      <c r="A45" s="13" t="inlineStr">
+      <c r="A45" s="15" t="inlineStr">
         <is>
           <t>Belgien vs Ägypten (15.06.)</t>
         </is>
       </c>
-      <c r="B45" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C45" s="15" t="inlineStr">
+      <c r="B45" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C45" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="D45" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E45" s="15" t="inlineStr">
+      <c r="E45" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F45" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="46">
-      <c r="A46" s="13" t="inlineStr">
+      <c r="A46" s="15" t="inlineStr">
         <is>
           <t>Iran vs Neuseeland (16.06.)</t>
         </is>
       </c>
-      <c r="B46" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C46" s="15" t="inlineStr">
+      <c r="B46" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C46" s="17" t="inlineStr">
+        <is>
+          <t>4:4</t>
+        </is>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D46" s="15" t="inlineStr">
+      <c r="E46" s="17" t="inlineStr">
         <is>
           <t>1:21</t>
         </is>
       </c>
-      <c r="E46" s="15" t="inlineStr">
+      <c r="F46" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="47">
-      <c r="A47" s="13" t="inlineStr">
+      <c r="A47" s="15" t="inlineStr">
         <is>
           <t>Belgien vs Iran (21.06.)</t>
         </is>
       </c>
-      <c r="B47" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C47" s="15" t="inlineStr">
+      <c r="B47" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C47" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D47" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D47" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E47" s="15" t="inlineStr">
+      <c r="E47" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F47" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="48">
-      <c r="A48" s="13" t="inlineStr">
+      <c r="A48" s="15" t="inlineStr">
         <is>
           <t>Neuseeland vs Ägypten (22.06.)</t>
         </is>
       </c>
-      <c r="B48" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C48" s="15" t="inlineStr">
+      <c r="B48" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C48" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D48" s="17" t="inlineStr">
         <is>
           <t>8:5</t>
         </is>
       </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E48" s="15" t="inlineStr">
+      <c r="E48" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F48" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="49">
-      <c r="A49" s="13" t="inlineStr">
+      <c r="A49" s="15" t="inlineStr">
         <is>
           <t>Ägypten vs Iran (27.06.)</t>
         </is>
       </c>
-      <c r="B49" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C49" s="15" t="inlineStr">
+      <c r="B49" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C49" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D49" s="17" t="inlineStr">
         <is>
           <t>5:4</t>
         </is>
       </c>
-      <c r="D49" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E49" s="15" t="inlineStr">
+      <c r="E49" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F49" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="13" t="inlineStr">
+      <c r="A50" s="15" t="inlineStr">
         <is>
           <t>Neuseeland vs Belgien (27.06.)</t>
         </is>
       </c>
-      <c r="B50" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C50" s="15" t="inlineStr">
+      <c r="B50" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C50" s="17" t="inlineStr">
+        <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="D50" s="17" t="inlineStr">
         <is>
           <t>8:5</t>
         </is>
       </c>
-      <c r="D50" s="15" t="inlineStr">
+      <c r="E50" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="E50" s="15" t="inlineStr">
+      <c r="F50" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="12" t="inlineStr">
+      <c r="A51" s="14" t="inlineStr">
         <is>
           <t>── Gruppe H ──</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="13" t="inlineStr">
+      <c r="A52" s="15" t="inlineStr">
         <is>
           <t>Spanien vs Kap Verde (15.06.)</t>
         </is>
       </c>
-      <c r="B52" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C52" s="15" t="inlineStr">
+      <c r="B52" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C52" s="17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="D52" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E52" s="15" t="inlineStr">
+      <c r="E52" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F52" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="53">
-      <c r="A53" s="13" t="inlineStr">
+      <c r="A53" s="15" t="inlineStr">
         <is>
           <t>Saudi-Arabien vs Uruguay (16.06.)</t>
         </is>
       </c>
-      <c r="B53" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C53" s="15" t="inlineStr">
+      <c r="B53" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C53" s="17" t="inlineStr">
+        <is>
+          <t>2:5</t>
+        </is>
+      </c>
+      <c r="D53" s="17" t="inlineStr">
         <is>
           <t>8:5</t>
         </is>
       </c>
-      <c r="D53" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E53" s="15" t="inlineStr">
+      <c r="E53" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="54">
-      <c r="A54" s="13" t="inlineStr">
+      <c r="A54" s="15" t="inlineStr">
         <is>
           <t>Spanien vs Saudi-Arabien (21.06.)</t>
         </is>
       </c>
-      <c r="B54" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C54" s="15" t="inlineStr">
+      <c r="B54" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C54" s="17" t="inlineStr">
+        <is>
+          <t>3:3</t>
+        </is>
+      </c>
+      <c r="D54" s="17" t="inlineStr">
         <is>
           <t>4:5</t>
         </is>
       </c>
-      <c r="D54" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E54" s="15" t="inlineStr">
+      <c r="E54" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F54" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="55">
-      <c r="A55" s="13" t="inlineStr">
+      <c r="A55" s="15" t="inlineStr">
         <is>
           <t>Uruguay vs Kap Verde (22.06.)</t>
         </is>
       </c>
-      <c r="B55" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C55" s="15" t="inlineStr">
+      <c r="B55" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C55" s="17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="D55" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D55" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E55" s="15" t="inlineStr">
+      <c r="E55" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F55" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="56">
-      <c r="A56" s="13" t="inlineStr">
+      <c r="A56" s="15" t="inlineStr">
         <is>
           <t>Kap Verde vs Saudi-Arabien (27.06.)</t>
         </is>
       </c>
-      <c r="B56" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C56" s="15" t="inlineStr">
+      <c r="B56" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C56" s="17" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="D56" s="17" t="inlineStr">
         <is>
           <t>2:8</t>
         </is>
       </c>
-      <c r="D56" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E56" s="15" t="inlineStr">
+      <c r="E56" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F56" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="57">
-      <c r="A57" s="13" t="inlineStr">
+      <c r="A57" s="15" t="inlineStr">
         <is>
           <t>Uruguay vs Spanien (27.06.)</t>
         </is>
       </c>
-      <c r="B57" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C57" s="15" t="inlineStr">
+      <c r="B57" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D57" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D57" s="15" t="inlineStr">
+      <c r="E57" s="17" t="inlineStr">
         <is>
           <t>1:21</t>
         </is>
       </c>
-      <c r="E57" s="15" t="inlineStr">
+      <c r="F57" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="58">
-      <c r="A58" s="12" t="inlineStr">
+      <c r="A58" s="14" t="inlineStr">
         <is>
           <t>── Gruppe I ──</t>
         </is>
       </c>
     </row>
     <row r="59">
-      <c r="A59" s="13" t="inlineStr">
+      <c r="A59" s="15" t="inlineStr">
         <is>
           <t>Frankreich vs Senegal (16.06.)</t>
         </is>
       </c>
-      <c r="B59" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C59" s="15" t="inlineStr">
+      <c r="B59" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D59" s="17" t="inlineStr">
         <is>
           <t>2:4</t>
         </is>
       </c>
-      <c r="D59" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E59" s="15" t="inlineStr">
+      <c r="E59" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="60">
-      <c r="A60" s="13" t="inlineStr">
+      <c r="A60" s="15" t="inlineStr">
         <is>
           <t>Irak vs Norwegen (17.06.)</t>
         </is>
       </c>
-      <c r="B60" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C60" s="15" t="inlineStr">
+      <c r="B60" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C60" s="17" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="D60" s="17" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="D60" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E60" s="15" t="inlineStr">
+      <c r="E60" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F60" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="13" t="inlineStr">
+      <c r="A61" s="15" t="inlineStr">
         <is>
           <t>Frankreich vs Irak (22.06.)</t>
         </is>
       </c>
-      <c r="B61" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C61" s="15" t="inlineStr">
+      <c r="B61" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C61" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D61" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D61" s="15" t="inlineStr">
+      <c r="E61" s="17" t="inlineStr">
         <is>
           <t>1:21</t>
         </is>
       </c>
-      <c r="E61" s="15" t="inlineStr">
+      <c r="F61" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="62">
-      <c r="A62" s="13" t="inlineStr">
+      <c r="A62" s="15" t="inlineStr">
         <is>
           <t>Norwegen vs Senegal (23.06.)</t>
         </is>
       </c>
-      <c r="B62" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C62" s="15" t="inlineStr">
+      <c r="B62" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C62" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D62" s="17" t="inlineStr">
         <is>
           <t>8:2</t>
         </is>
       </c>
-      <c r="D62" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E62" s="15" t="inlineStr">
+      <c r="E62" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F62" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="63">
-      <c r="A63" s="13" t="inlineStr">
+      <c r="A63" s="15" t="inlineStr">
         <is>
           <t>Norwegen vs Frankreich (26.06.)</t>
         </is>
       </c>
-      <c r="B63" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C63" s="15" t="inlineStr">
+      <c r="B63" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C63" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D63" s="17" t="inlineStr">
         <is>
           <t>4:28</t>
         </is>
       </c>
-      <c r="D63" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E63" s="15" t="inlineStr">
+      <c r="E63" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F63" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="64">
-      <c r="A64" s="13" t="inlineStr">
+      <c r="A64" s="15" t="inlineStr">
         <is>
           <t>Senegal vs Irak (26.06.)</t>
         </is>
       </c>
-      <c r="B64" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C64" s="15" t="inlineStr">
+      <c r="B64" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C64" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D64" s="17" t="inlineStr">
         <is>
           <t>8:4</t>
         </is>
       </c>
-      <c r="D64" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E64" s="15" t="inlineStr">
+      <c r="E64" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F64" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="65">
-      <c r="A65" s="12" t="inlineStr">
+      <c r="A65" s="14" t="inlineStr">
         <is>
           <t>── Gruppe J ──</t>
         </is>
       </c>
     </row>
     <row r="66">
-      <c r="A66" s="13" t="inlineStr">
+      <c r="A66" s="15" t="inlineStr">
         <is>
           <t>Argentinien vs Algerien (17.06.)</t>
         </is>
       </c>
-      <c r="B66" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C66" s="15" t="inlineStr">
+      <c r="B66" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D66" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D66" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E66" s="15" t="inlineStr">
+      <c r="E66" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F66" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="67">
-      <c r="A67" s="13" t="inlineStr">
+      <c r="A67" s="15" t="inlineStr">
         <is>
           <t>Österreich vs Jordanien (17.06.)</t>
         </is>
       </c>
-      <c r="B67" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C67" s="15" t="inlineStr">
+      <c r="B67" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C67" s="17" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="D67" s="17" t="inlineStr">
         <is>
           <t>4:8</t>
         </is>
       </c>
-      <c r="D67" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E67" s="15" t="inlineStr">
+      <c r="E67" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F67" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="68">
-      <c r="A68" s="13" t="inlineStr">
+      <c r="A68" s="15" t="inlineStr">
         <is>
           <t>Argentinien vs Österreich (22.06.)</t>
         </is>
       </c>
-      <c r="B68" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C68" s="15" t="inlineStr">
+      <c r="B68" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C68" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D68" s="17" t="inlineStr">
         <is>
           <t>2:4</t>
         </is>
       </c>
-      <c r="D68" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E68" s="15" t="inlineStr">
+      <c r="E68" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F68" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="13" t="inlineStr">
+      <c r="A69" s="15" t="inlineStr">
         <is>
           <t>Jordanien vs Algerien (23.06.)</t>
         </is>
       </c>
-      <c r="B69" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C69" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D69" s="15" t="inlineStr">
+      <c r="B69" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D69" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E69" s="15" t="inlineStr">
+      <c r="F69" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="70">
-      <c r="A70" s="13" t="inlineStr">
+      <c r="A70" s="15" t="inlineStr">
         <is>
           <t>Algerien vs Österreich (28.06.)</t>
         </is>
       </c>
-      <c r="B70" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C70" s="15" t="inlineStr">
+      <c r="B70" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C70" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D70" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="D70" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E70" s="15" t="inlineStr">
+      <c r="E70" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F70" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
     </row>
     <row r="71">
-      <c r="A71" s="13" t="inlineStr">
+      <c r="A71" s="15" t="inlineStr">
         <is>
           <t>Jordanien vs Argentinien (28.06.)</t>
         </is>
       </c>
-      <c r="B71" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C71" s="15" t="inlineStr">
+      <c r="B71" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C71" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="D71" s="17" t="inlineStr">
         <is>
           <t>1:5</t>
         </is>
       </c>
-      <c r="D71" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E71" s="15" t="inlineStr">
+      <c r="E71" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F71" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="12" t="inlineStr">
+      <c r="A72" s="14" t="inlineStr">
         <is>
           <t>── Gruppe K ──</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="13" t="inlineStr">
+      <c r="A73" s="15" t="inlineStr">
         <is>
           <t>Portugal vs DR Kongo (17.06.)</t>
         </is>
       </c>
-      <c r="B73" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C73" s="15" t="inlineStr">
+      <c r="B73" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C73" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D73" s="17" t="inlineStr">
         <is>
           <t>5:1</t>
         </is>
       </c>
-      <c r="D73" s="15" t="inlineStr">
+      <c r="E73" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E73" s="15" t="inlineStr">
+      <c r="F73" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="13" t="inlineStr">
+      <c r="A74" s="15" t="inlineStr">
         <is>
           <t>Usbekistan vs Kolumbien (18.06.)</t>
         </is>
       </c>
-      <c r="B74" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C74" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D74" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E74" s="15" t="inlineStr">
+      <c r="B74" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C74" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D74" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E74" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F74" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="75">
-      <c r="A75" s="13" t="inlineStr">
+      <c r="A75" s="15" t="inlineStr">
         <is>
           <t>Portugal vs Usbekistan (23.06.)</t>
         </is>
       </c>
-      <c r="B75" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C75" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D75" s="15" t="inlineStr">
+      <c r="B75" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C75" s="17" t="inlineStr">
+        <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="D75" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E75" s="17" t="inlineStr">
         <is>
           <t>1:21</t>
         </is>
       </c>
-      <c r="E75" s="15" t="inlineStr">
+      <c r="F75" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="76">
-      <c r="A76" s="13" t="inlineStr">
+      <c r="A76" s="15" t="inlineStr">
         <is>
           <t>Kolumbien vs DR Kongo (24.06.)</t>
         </is>
       </c>
-      <c r="B76" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C76" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D76" s="15" t="inlineStr">
+      <c r="B76" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C76" s="17" t="inlineStr">
+        <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="D76" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E76" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E76" s="15" t="inlineStr">
+      <c r="F76" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="77">
-      <c r="A77" s="13" t="inlineStr">
+      <c r="A77" s="15" t="inlineStr">
         <is>
           <t>Kolumbien vs Portugal (28.06.)</t>
         </is>
       </c>
-      <c r="B77" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C77" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D77" s="15" t="inlineStr">
+      <c r="B77" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C77" s="17" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="D77" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E77" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E77" s="15" t="inlineStr">
+      <c r="F77" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="78">
-      <c r="A78" s="13" t="inlineStr">
+      <c r="A78" s="15" t="inlineStr">
         <is>
           <t>DR Kongo vs Usbekistan (28.06.)</t>
         </is>
       </c>
-      <c r="B78" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C78" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D78" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E78" s="15" t="inlineStr">
+      <c r="B78" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C78" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D78" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E78" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F78" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="79">
-      <c r="A79" s="12" t="inlineStr">
+      <c r="A79" s="14" t="inlineStr">
         <is>
           <t>── Gruppe L ──</t>
         </is>
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="13" t="inlineStr">
+      <c r="A80" s="15" t="inlineStr">
         <is>
           <t>England vs Kroatien (17.06.)</t>
         </is>
       </c>
-      <c r="B80" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C80" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D80" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E80" s="15" t="inlineStr">
+      <c r="B80" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C80" s="17" t="inlineStr">
+        <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="D80" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E80" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F80" s="17" t="inlineStr">
         <is>
           <t>2:12</t>
         </is>
       </c>
     </row>
     <row r="81">
-      <c r="A81" s="13" t="inlineStr">
+      <c r="A81" s="15" t="inlineStr">
         <is>
           <t>Ghana vs Panama (18.06.)</t>
         </is>
       </c>
-      <c r="B81" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C81" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D81" s="15" t="inlineStr">
+      <c r="B81" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C81" s="17" t="inlineStr">
+        <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="D81" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E81" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="E81" s="15" t="inlineStr">
+      <c r="F81" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="13" t="inlineStr">
+      <c r="A82" s="15" t="inlineStr">
         <is>
           <t>England vs Ghana (23.06.)</t>
         </is>
       </c>
-      <c r="B82" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C82" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D82" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E82" s="15" t="inlineStr">
+      <c r="B82" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C82" s="17" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="D82" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E82" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F82" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="83">
-      <c r="A83" s="13" t="inlineStr">
+      <c r="A83" s="15" t="inlineStr">
         <is>
           <t>Panama vs Kroatien (24.06.)</t>
         </is>
       </c>
-      <c r="B83" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C83" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="D83" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E83" s="15" t="inlineStr">
+      <c r="B83" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C83" s="17" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="D83" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="E83" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F83" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="84">
-      <c r="A84" s="13" t="inlineStr">
+      <c r="A84" s="15" t="inlineStr">
         <is>
           <t>Panama vs England (27.06.)</t>
         </is>
       </c>
-      <c r="B84" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C84" s="15" t="inlineStr">
+      <c r="B84" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C84" s="17" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="D84" s="17" t="inlineStr">
         <is>
           <t>2:21</t>
         </is>
       </c>
-      <c r="D84" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E84" s="15" t="inlineStr">
+      <c r="E84" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F84" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
       </c>
     </row>
     <row r="85">
-      <c r="A85" s="13" t="inlineStr">
+      <c r="A85" s="15" t="inlineStr">
         <is>
           <t>Kroatien vs Ghana (27.06.)</t>
         </is>
       </c>
-      <c r="B85" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C85" s="15" t="inlineStr">
+      <c r="B85" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C85" s="17" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="D85" s="17" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="D85" s="15" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="E85" s="15" t="inlineStr">
+      <c r="E85" s="17" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="F85" s="17" t="inlineStr">
         <is>
           <t>2:1</t>
         </is>
@@ -2786,18 +3195,18 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A30:E30"/>
-    <mergeCell ref="A65:E65"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A16:E16"/>
-    <mergeCell ref="A72:E72"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A37:E37"/>
-    <mergeCell ref="A44:E44"/>
-    <mergeCell ref="A58:E58"/>
-    <mergeCell ref="A9:E9"/>
-    <mergeCell ref="A79:E79"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A51:F51"/>
+    <mergeCell ref="A44:F44"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A37:F37"/>
+    <mergeCell ref="A79:F79"/>
+    <mergeCell ref="A58:F58"/>
+    <mergeCell ref="A30:F30"/>
+    <mergeCell ref="A72:F72"/>
+    <mergeCell ref="A65:F65"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2809,7 +3218,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E37"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2817,902 +3226,1063 @@
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="10" t="inlineStr">
+      <c r="A1" s="12" t="inlineStr">
         <is>
           <t>KO-Runde / Slot</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="12" t="inlineStr">
         <is>
           <t>Tatsächlich</t>
         </is>
       </c>
-      <c r="C1" s="11" t="inlineStr">
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>italien</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
         <is>
           <t>Timo Test1</t>
         </is>
       </c>
-      <c r="D1" s="11" t="inlineStr">
+      <c r="E1" s="13" t="inlineStr">
         <is>
           <t>Timo Test2</t>
         </is>
       </c>
-      <c r="E1" s="11" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Timo Test3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="14" t="inlineStr">
         <is>
           <t>── Achtelfinale-Teilnehmer (16) (je 5 Pkt.) ──</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 1</t>
         </is>
       </c>
-      <c r="B3" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C3" s="15" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C3" s="17" t="inlineStr">
+        <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="D3" s="17" t="inlineStr">
         <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="D3" s="15" t="inlineStr">
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>Kanada</t>
         </is>
       </c>
-      <c r="E3" s="15" t="inlineStr">
+      <c r="F3" s="17" t="inlineStr">
         <is>
           <t>Kanada</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="13" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 2</t>
         </is>
       </c>
-      <c r="B4" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C4" s="15" t="inlineStr">
+      <c r="B4" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Haiti</t>
+        </is>
+      </c>
+      <c r="D4" s="17" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="D4" s="15" t="inlineStr">
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Marokko</t>
         </is>
       </c>
-      <c r="E4" s="15" t="inlineStr">
+      <c r="F4" s="17" t="inlineStr">
         <is>
           <t>Marokko</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="13" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 3</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C5" s="15" t="inlineStr">
+      <c r="B5" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C5" s="17" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="D5" s="17" t="inlineStr">
         <is>
           <t>Elfenbeinküste</t>
         </is>
       </c>
-      <c r="D5" s="15" t="inlineStr">
+      <c r="E5" s="17" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="E5" s="15" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="13" t="inlineStr">
+      <c r="A6" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 4</t>
         </is>
       </c>
-      <c r="B6" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C6" s="15" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C6" s="17" t="inlineStr">
+        <is>
+          <t>Schweden</t>
+        </is>
+      </c>
+      <c r="D6" s="17" t="inlineStr">
         <is>
           <t>Japan</t>
         </is>
       </c>
-      <c r="D6" s="15" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>Schweden</t>
         </is>
       </c>
-      <c r="E6" s="15" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="13" t="inlineStr">
+      <c r="A7" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 5</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C7" s="15" t="inlineStr">
+      <c r="B7" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="D7" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="D7" s="15" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>Ecuador</t>
         </is>
       </c>
-      <c r="E7" s="15" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Ecuador</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="13" t="inlineStr">
+      <c r="A8" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 6</t>
         </is>
       </c>
-      <c r="B8" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C8" s="15" t="inlineStr">
+      <c r="B8" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C8" s="17" t="inlineStr">
+        <is>
+          <t>Senegal</t>
+        </is>
+      </c>
+      <c r="D8" s="17" t="inlineStr">
         <is>
           <t>Iran</t>
         </is>
       </c>
-      <c r="D8" s="15" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>Schottland</t>
         </is>
       </c>
-      <c r="E8" s="15" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>Australien</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="13" t="inlineStr">
+      <c r="A9" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 7</t>
         </is>
       </c>
-      <c r="B9" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C9" s="15" t="inlineStr">
+      <c r="B9" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C9" s="17" t="inlineStr">
+        <is>
+          <t>Tschechien</t>
+        </is>
+      </c>
+      <c r="D9" s="17" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="D9" s="15" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>Mexiko</t>
         </is>
       </c>
-      <c r="E9" s="15" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Mexiko</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 8</t>
         </is>
       </c>
-      <c r="B10" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C10" s="15" t="inlineStr">
+      <c r="B10" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C10" s="17" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+      <c r="D10" s="17" t="inlineStr">
         <is>
           <t>Usbekistan</t>
         </is>
       </c>
-      <c r="D10" s="15" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>Panama</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 9</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C11" s="15" t="inlineStr">
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C11" s="17" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="D11" s="17" t="inlineStr">
         <is>
           <t>Südkorea</t>
         </is>
       </c>
-      <c r="D11" s="15" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="E11" s="15" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 10</t>
         </is>
       </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C12" s="15" t="inlineStr">
+      <c r="B12" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C12" s="17" t="inlineStr">
+        <is>
+          <t>Türkei</t>
+        </is>
+      </c>
+      <c r="D12" s="17" t="inlineStr">
         <is>
           <t>Australien</t>
         </is>
       </c>
-      <c r="D12" s="15" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="E12" s="15" t="inlineStr">
+      <c r="F12" s="17" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 11</t>
         </is>
       </c>
-      <c r="B13" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C13" s="17" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="D13" s="17" t="inlineStr">
         <is>
           <t>Österreich</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="F13" s="17" t="inlineStr">
         <is>
           <t>Jordanien</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 12</t>
         </is>
       </c>
-      <c r="B14" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="B14" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C14" s="17" t="inlineStr">
+        <is>
+          <t>Usbekistan</t>
+        </is>
+      </c>
+      <c r="D14" s="17" t="inlineStr">
         <is>
           <t>Kolumbien</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="E14" s="17" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="F14" s="17" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 13</t>
         </is>
       </c>
-      <c r="B15" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="B15" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
         <is>
           <t>Kanada</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D15" s="17" t="inlineStr">
+        <is>
+          <t>Kanada</t>
+        </is>
+      </c>
+      <c r="E15" s="17" t="inlineStr">
         <is>
           <t>Ägypten</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="F15" s="17" t="inlineStr">
         <is>
           <t>Bosnien-Herzegowina</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 14</t>
         </is>
       </c>
-      <c r="B16" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C16" s="15" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C16" s="17" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D16" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D16" s="15" t="inlineStr">
+      <c r="E16" s="17" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
-      <c r="E16" s="15" t="inlineStr">
+      <c r="F16" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 15</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C17" s="15" t="inlineStr">
+      <c r="B17" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C17" s="17" t="inlineStr">
+        <is>
+          <t>Österreich</t>
+        </is>
+      </c>
+      <c r="D17" s="17" t="inlineStr">
         <is>
           <t>Jordanien</t>
         </is>
       </c>
-      <c r="D17" s="15" t="inlineStr">
+      <c r="E17" s="17" t="inlineStr">
         <is>
           <t>Algerien</t>
         </is>
       </c>
-      <c r="E17" s="15" t="inlineStr">
+      <c r="F17" s="17" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 16</t>
         </is>
       </c>
-      <c r="B18" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C18" s="15" t="inlineStr">
+      <c r="B18" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C18" s="17" t="inlineStr">
+        <is>
+          <t>Kolumbien</t>
+        </is>
+      </c>
+      <c r="D18" s="17" t="inlineStr">
         <is>
           <t>Irak</t>
         </is>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="E18" s="17" t="inlineStr">
         <is>
           <t>Paraguay</t>
         </is>
       </c>
-      <c r="E18" s="15" t="inlineStr">
+      <c r="F18" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>── Viertelfinale-Teilnehmer (8) (je 10 Pkt.) ──</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 1</t>
         </is>
       </c>
-      <c r="B20" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C20" s="15" t="inlineStr">
+      <c r="B20" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C20" s="17" t="inlineStr">
+        <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="D20" s="17" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="D20" s="15" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Marokko</t>
         </is>
       </c>
-      <c r="E20" s="15" t="inlineStr">
+      <c r="F20" s="17" t="inlineStr">
         <is>
           <t>Marokko</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 2</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C21" s="15" t="inlineStr">
+      <c r="B21" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
         <is>
           <t>Elfenbeinküste</t>
         </is>
       </c>
-      <c r="D21" s="15" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="E21" s="15" t="inlineStr">
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 3</t>
         </is>
       </c>
-      <c r="B22" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C22" s="15" t="inlineStr">
+      <c r="B22" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C22" s="17" t="inlineStr">
+        <is>
+          <t>Ecuador</t>
+        </is>
+      </c>
+      <c r="D22" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="D22" s="15" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>Schottland</t>
         </is>
       </c>
-      <c r="E22" s="15" t="inlineStr">
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>Australien</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 4</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C23" s="15" t="inlineStr">
+      <c r="B23" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C23" s="17" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+      <c r="D23" s="17" t="inlineStr">
         <is>
           <t>Uruguay</t>
         </is>
       </c>
-      <c r="D23" s="15" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>Mexiko</t>
         </is>
       </c>
-      <c r="E23" s="15" t="inlineStr">
+      <c r="F23" s="17" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 5</t>
         </is>
       </c>
-      <c r="B24" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="B24" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C24" s="17" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="D24" s="17" t="inlineStr">
         <is>
           <t>Südkorea</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
+      <c r="E24" s="17" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="E24" s="15" t="inlineStr">
+      <c r="F24" s="17" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 6</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C25" s="15" t="inlineStr">
+      <c r="B25" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>Uruguay</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>Österreich</t>
         </is>
       </c>
-      <c r="D25" s="15" t="inlineStr">
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="E25" s="15" t="inlineStr">
+      <c r="F25" s="17" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 7</t>
         </is>
       </c>
-      <c r="B26" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="B26" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C26" s="17" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D26" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
+      <c r="E26" s="17" t="inlineStr">
         <is>
           <t>Ägypten</t>
         </is>
       </c>
-      <c r="E26" s="15" t="inlineStr">
+      <c r="F26" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 8</t>
         </is>
       </c>
-      <c r="B27" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C27" s="15" t="inlineStr">
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C27" s="17" t="inlineStr">
+        <is>
+          <t>Österreich</t>
+        </is>
+      </c>
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>Irak</t>
         </is>
       </c>
-      <c r="D27" s="15" t="inlineStr">
+      <c r="E27" s="17" t="inlineStr">
         <is>
           <t>Algerien</t>
         </is>
       </c>
-      <c r="E27" s="15" t="inlineStr">
+      <c r="F27" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>── Halbfinale-Teilnehmer (4) (je 15 Pkt.) ──</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 1</t>
         </is>
       </c>
-      <c r="B29" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
+      <c r="B29" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C29" s="17" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="D29" s="17" t="inlineStr">
         <is>
           <t>Elfenbeinküste</t>
         </is>
       </c>
-      <c r="D29" s="15" t="inlineStr">
+      <c r="E29" s="17" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="E29" s="15" t="inlineStr">
+      <c r="F29" s="17" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+      <c r="A30" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 2</t>
         </is>
       </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
+      <c r="B30" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C30" s="17" t="inlineStr">
+        <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="E30" s="17" t="inlineStr">
         <is>
           <t>Schottland</t>
         </is>
       </c>
-      <c r="E30" s="15" t="inlineStr">
+      <c r="F30" s="17" t="inlineStr">
         <is>
           <t>Australien</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="13" t="inlineStr">
+      <c r="A31" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 3</t>
         </is>
       </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C31" s="15" t="inlineStr">
+      <c r="B31" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="D31" s="17" t="inlineStr">
         <is>
           <t>Südkorea</t>
         </is>
       </c>
-      <c r="D31" s="15" t="inlineStr">
+      <c r="E31" s="17" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="E31" s="15" t="inlineStr">
+      <c r="F31" s="17" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="13" t="inlineStr">
+      <c r="A32" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 4</t>
         </is>
       </c>
-      <c r="B32" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
+      <c r="B32" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C32" s="17" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="D32" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D32" s="15" t="inlineStr">
+      <c r="E32" s="17" t="inlineStr">
         <is>
           <t>Ägypten</t>
         </is>
       </c>
-      <c r="E32" s="15" t="inlineStr">
+      <c r="F32" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="A33" s="14" t="inlineStr">
         <is>
           <t>── Finale (je 20 Pkt.) ──</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="13" t="inlineStr">
+      <c r="A34" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 1</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
+      <c r="B34" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C34" s="17" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="D34" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
-      <c r="D34" s="15" t="inlineStr">
+      <c r="E34" s="17" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="E34" s="15" t="inlineStr">
+      <c r="F34" s="17" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="13" t="inlineStr">
+      <c r="A35" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 2</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C35" s="15" t="inlineStr">
+      <c r="B35" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C35" s="17" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D35" s="15" t="inlineStr">
+      <c r="E35" s="17" t="inlineStr">
         <is>
           <t>Ägypten</t>
         </is>
       </c>
-      <c r="E35" s="15" t="inlineStr">
+      <c r="F35" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="12" t="inlineStr">
+      <c r="A36" s="14" t="inlineStr">
         <is>
           <t>── Weltmeister (je 25 Pkt.) ──</t>
         </is>
       </c>
     </row>
     <row r="37">
-      <c r="A37" s="13" t="inlineStr">
+      <c r="A37" s="15" t="inlineStr">
         <is>
           <t xml:space="preserve">  Weiterkommer 1</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
-        <is>
-          <t>–</t>
-        </is>
-      </c>
-      <c r="C37" s="15" t="inlineStr">
+      <c r="B37" s="16" t="inlineStr">
+        <is>
+          <t>–</t>
+        </is>
+      </c>
+      <c r="C37" s="17" t="inlineStr">
+        <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="D37" s="17" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="D37" s="15" t="inlineStr">
+      <c r="E37" s="17" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="E37" s="15" t="inlineStr">
+      <c r="F37" s="17" t="inlineStr">
         <is>
           <t>Curaçao</t>
         </is>
@@ -3720,11 +4290,11 @@
     </row>
   </sheetData>
   <mergeCells count="5">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A33:E33"/>
-    <mergeCell ref="A19:E19"/>
-    <mergeCell ref="A36:E36"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A33:F33"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="A19:F19"/>
+    <mergeCell ref="A36:F36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix Scoring: HF (Finalisten +20/Team) korrekt berechnet; Finale-Doppelzählung entfernt; HF-Spalte in Rangliste aktiv
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -535,7 +535,7 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
@@ -583,12 +583,12 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
+          <t>Finalisten (+20)</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
           <t>Platz 3</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>Finale</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
@@ -3626,7 +3626,7 @@
     <row r="33">
       <c r="A33" s="12" t="inlineStr">
         <is>
-          <t>── Finale (je 20 Pkt.) ──</t>
+          <t>── Finalisten (2) (je 20 Pkt.) ──</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rony Burkart: neuer Tippzettel (WM-Tipp: Deutschland)
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -6251,7 +6251,7 @@
       </c>
       <c r="K4" s="17" t="inlineStr">
         <is>
-          <t>Niederlande</t>
+          <t>Brasilien</t>
         </is>
       </c>
       <c r="L4" s="17" t="inlineStr">
@@ -7263,7 +7263,7 @@
       </c>
       <c r="K20" s="17" t="inlineStr">
         <is>
-          <t>Niederlande</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="L20" s="17" t="inlineStr">
@@ -7330,7 +7330,7 @@
       </c>
       <c r="K21" s="17" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>Mexiko</t>
         </is>
       </c>
       <c r="L21" s="17" t="inlineStr">
@@ -7397,7 +7397,7 @@
       </c>
       <c r="K22" s="17" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Brasilien</t>
         </is>
       </c>
       <c r="L22" s="17" t="inlineStr">
@@ -7531,7 +7531,7 @@
       </c>
       <c r="K24" s="17" t="inlineStr">
         <is>
-          <t>Belgien</t>
+          <t>Spanien</t>
         </is>
       </c>
       <c r="L24" s="17" t="inlineStr">
@@ -7598,7 +7598,7 @@
       </c>
       <c r="K25" s="17" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>Türkei</t>
         </is>
       </c>
       <c r="L25" s="17" t="inlineStr">
@@ -7665,7 +7665,7 @@
       </c>
       <c r="K26" s="17" t="inlineStr">
         <is>
-          <t>Schweiz</t>
+          <t>Argentinien</t>
         </is>
       </c>
       <c r="L26" s="17" t="inlineStr">
@@ -7873,7 +7873,7 @@
       </c>
       <c r="K30" s="17" t="inlineStr">
         <is>
-          <t>Frankreich</t>
+          <t>Spanien</t>
         </is>
       </c>
       <c r="L30" s="17" t="inlineStr">
@@ -7940,7 +7940,7 @@
       </c>
       <c r="K31" s="17" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>England</t>
         </is>
       </c>
       <c r="L31" s="17" t="inlineStr">
@@ -8148,7 +8148,7 @@
       </c>
       <c r="K35" s="17" t="inlineStr">
         <is>
-          <t>Spanien</t>
+          <t>England</t>
         </is>
       </c>
       <c r="L35" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Live-Update: Kanada 0:1 Bosnien (45'+4')
</commit_message>
<xml_diff>
--- a/Rangliste.xlsx
+++ b/Rangliste.xlsx
@@ -826,14 +826,14 @@
       </c>
       <c r="B7" s="11" t="inlineStr">
         <is>
-          <t>Egon Hejda</t>
+          <t>Christian Sandritter</t>
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E7" s="7" t="n">
         <v>0</v>
@@ -863,7 +863,7 @@
       </c>
       <c r="B8" s="11" t="inlineStr">
         <is>
-          <t>Friedbert Mechler</t>
+          <t>Egon Hejda</t>
         </is>
       </c>
       <c r="C8" s="10" t="n">
@@ -900,7 +900,7 @@
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>Stefan Seiler</t>
+          <t>Friedbert Mechler</t>
         </is>
       </c>
       <c r="C9" s="10" t="n">
@@ -937,14 +937,14 @@
       </c>
       <c r="B10" s="11" t="inlineStr">
         <is>
-          <t>Heiko Baust</t>
+          <t>Rony Burkart</t>
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>0</v>
@@ -974,14 +974,14 @@
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>Christian Sandritter</t>
+          <t>Stefan Seiler</t>
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D11" s="7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E11" s="7" t="n">
         <v>0</v>
@@ -1011,14 +1011,14 @@
       </c>
       <c r="B12" s="11" t="inlineStr">
         <is>
-          <t>Markus Bruckner</t>
+          <t>Heiko Baust</t>
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D12" s="4" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>0</v>
@@ -1048,7 +1048,7 @@
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>Rony Burkart</t>
+          <t>Markus Bruckner</t>
         </is>
       </c>
       <c r="C13" s="10" t="n">
@@ -1147,37 +1147,37 @@
       </c>
       <c r="H1" s="13" t="inlineStr">
         <is>
+          <t>Christian Sandritter</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
           <t>Egon Hejda</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Friedbert Mechler</t>
         </is>
       </c>
-      <c r="J1" s="13" t="inlineStr">
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>Rony Burkart</t>
+        </is>
+      </c>
+      <c r="L1" s="13" t="inlineStr">
         <is>
           <t>Stefan Seiler</t>
         </is>
       </c>
-      <c r="K1" s="13" t="inlineStr">
+      <c r="M1" s="13" t="inlineStr">
         <is>
           <t>Heiko Baust</t>
         </is>
       </c>
-      <c r="L1" s="13" t="inlineStr">
-        <is>
-          <t>Christian Sandritter</t>
-        </is>
-      </c>
-      <c r="M1" s="13" t="inlineStr">
+      <c r="N1" s="13" t="inlineStr">
         <is>
           <t>Markus Bruckner</t>
-        </is>
-      </c>
-      <c r="N1" s="13" t="inlineStr">
-        <is>
-          <t>Rony Burkart</t>
         </is>
       </c>
     </row>
@@ -1224,39 +1224,39 @@
           <t>3:1  (+3)</t>
         </is>
       </c>
-      <c r="H3" s="17" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
+        <is>
+          <t>2:1  (+2)</t>
+        </is>
+      </c>
+      <c r="I3" s="17" t="inlineStr">
         <is>
           <t>2:0  (+4)</t>
         </is>
       </c>
-      <c r="I3" s="17" t="inlineStr">
+      <c r="J3" s="17" t="inlineStr">
         <is>
           <t>2:0  (+4)</t>
         </is>
       </c>
-      <c r="J3" s="17" t="inlineStr">
+      <c r="K3" s="18" t="inlineStr">
+        <is>
+          <t>1:0  (+2)</t>
+        </is>
+      </c>
+      <c r="L3" s="17" t="inlineStr">
         <is>
           <t>2:0  (+4)</t>
         </is>
       </c>
-      <c r="K3" s="19" t="inlineStr">
+      <c r="M3" s="19" t="inlineStr">
         <is>
           <t>3:1  (+3)</t>
         </is>
       </c>
-      <c r="L3" s="18" t="inlineStr">
+      <c r="N3" s="18" t="inlineStr">
         <is>
           <t>2:1  (+2)</t>
-        </is>
-      </c>
-      <c r="M3" s="18" t="inlineStr">
-        <is>
-          <t>2:1  (+2)</t>
-        </is>
-      </c>
-      <c r="N3" s="18" t="inlineStr">
-        <is>
-          <t>1:0  (+2)</t>
         </is>
       </c>
     </row>
@@ -1298,37 +1298,37 @@
       </c>
       <c r="H4" s="20" t="inlineStr">
         <is>
+          <t>1:1  (+0)</t>
+        </is>
+      </c>
+      <c r="I4" s="20" t="inlineStr">
+        <is>
           <t>0:0  (+0)</t>
         </is>
       </c>
-      <c r="I4" s="20" t="inlineStr">
+      <c r="J4" s="20" t="inlineStr">
         <is>
           <t>1:1  (+0)</t>
         </is>
       </c>
-      <c r="J4" s="20" t="inlineStr">
+      <c r="K4" s="20" t="inlineStr">
+        <is>
+          <t>0:3  (+0)</t>
+        </is>
+      </c>
+      <c r="L4" s="20" t="inlineStr">
         <is>
           <t>1:1  (+0)</t>
         </is>
       </c>
-      <c r="K4" s="20" t="inlineStr">
+      <c r="M4" s="20" t="inlineStr">
         <is>
           <t>1:3  (+0)</t>
         </is>
       </c>
-      <c r="L4" s="20" t="inlineStr">
-        <is>
-          <t>1:1  (+0)</t>
-        </is>
-      </c>
-      <c r="M4" s="20" t="inlineStr">
+      <c r="N4" s="20" t="inlineStr">
         <is>
           <t>1:2  (+0)</t>
-        </is>
-      </c>
-      <c r="N4" s="20" t="inlineStr">
-        <is>
-          <t>0:3  (+0)</t>
         </is>
       </c>
     </row>
@@ -1370,37 +1370,37 @@
       </c>
       <c r="H5" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I5" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I5" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J5" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K5" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L5" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="L5" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
       <c r="M5" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="N5" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
-        </is>
-      </c>
-      <c r="N5" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -1442,37 +1442,37 @@
       </c>
       <c r="H6" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="I6" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I6" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="J6" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="K6" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="L6" s="21" t="inlineStr">
+        <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="K6" s="21" t="inlineStr">
+      <c r="M6" s="21" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="L6" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="M6" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N6" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -1514,37 +1514,37 @@
       </c>
       <c r="H7" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I7" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="I7" s="21" t="inlineStr">
+      <c r="J7" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J7" s="21" t="inlineStr">
+      <c r="K7" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L7" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="L7" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
       <c r="M7" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N7" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
-        </is>
-      </c>
-      <c r="N7" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -1586,37 +1586,37 @@
       </c>
       <c r="H8" s="21" t="inlineStr">
         <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="I8" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="I8" s="21" t="inlineStr">
+      <c r="J8" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J8" s="21" t="inlineStr">
+      <c r="K8" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K8" s="21" t="inlineStr">
+      <c r="L8" s="21" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="M8" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="L8" s="21" t="inlineStr">
-        <is>
-          <t>0:1</t>
-        </is>
-      </c>
-      <c r="M8" s="21" t="inlineStr">
+      <c r="N8" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N8" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
         </is>
       </c>
     </row>
@@ -1665,37 +1665,37 @@
       </c>
       <c r="H10" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="I10" s="21" t="inlineStr">
+        <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="I10" s="21" t="inlineStr">
+      <c r="J10" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J10" s="21" t="inlineStr">
+      <c r="K10" s="21" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="L10" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K10" s="21" t="inlineStr">
+      <c r="M10" s="21" t="inlineStr">
         <is>
           <t>3:2</t>
         </is>
       </c>
-      <c r="L10" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M10" s="21" t="inlineStr">
+      <c r="N10" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N10" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
         </is>
       </c>
     </row>
@@ -1737,37 +1737,37 @@
       </c>
       <c r="H11" s="21" t="inlineStr">
         <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="I11" s="21" t="inlineStr">
+        <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="I11" s="21" t="inlineStr">
+      <c r="J11" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J11" s="21" t="inlineStr">
+      <c r="K11" s="21" t="inlineStr">
+        <is>
+          <t>0:4</t>
+        </is>
+      </c>
+      <c r="L11" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="K11" s="21" t="inlineStr">
+      <c r="M11" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="L11" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
-        </is>
-      </c>
-      <c r="M11" s="21" t="inlineStr">
+      <c r="N11" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
-        </is>
-      </c>
-      <c r="N11" s="21" t="inlineStr">
-        <is>
-          <t>0:4</t>
         </is>
       </c>
     </row>
@@ -1809,37 +1809,37 @@
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>3:2</t>
         </is>
       </c>
       <c r="I12" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="J12" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="J12" s="21" t="inlineStr">
+      <c r="K12" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L12" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="K12" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="L12" s="21" t="inlineStr">
-        <is>
-          <t>3:2</t>
-        </is>
-      </c>
       <c r="M12" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="N12" s="21" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -1881,37 +1881,37 @@
       </c>
       <c r="H13" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="I13" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="I13" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J13" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K13" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L13" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="K13" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="L13" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="M13" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N13" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N13" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -1953,37 +1953,37 @@
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
+          <t>4:1</t>
+        </is>
+      </c>
+      <c r="I14" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="I14" s="21" t="inlineStr">
+      <c r="J14" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="J14" s="21" t="inlineStr">
+      <c r="K14" s="21" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="L14" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K14" s="21" t="inlineStr">
+      <c r="M14" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="L14" s="21" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="M14" s="21" t="inlineStr">
+      <c r="N14" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
-        </is>
-      </c>
-      <c r="N14" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
         </is>
       </c>
     </row>
@@ -2025,7 +2025,7 @@
       </c>
       <c r="H15" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="I15" s="21" t="inlineStr">
@@ -2035,27 +2035,27 @@
       </c>
       <c r="J15" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K15" s="21" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="L15" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K15" s="21" t="inlineStr">
+      <c r="M15" s="21" t="inlineStr">
         <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="L15" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="M15" s="21" t="inlineStr">
+      <c r="N15" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N15" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
         </is>
       </c>
     </row>
@@ -2109,7 +2109,7 @@
       </c>
       <c r="I17" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="J17" s="21" t="inlineStr">
@@ -2119,22 +2119,22 @@
       </c>
       <c r="K17" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L17" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="M17" s="21" t="inlineStr">
+        <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="L17" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="M17" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="N17" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2191,22 +2191,22 @@
       </c>
       <c r="K18" s="21" t="inlineStr">
         <is>
+          <t>0:4</t>
+        </is>
+      </c>
+      <c r="L18" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="L18" s="21" t="inlineStr">
+      <c r="M18" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="M18" s="21" t="inlineStr">
+      <c r="N18" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
-        </is>
-      </c>
-      <c r="N18" s="21" t="inlineStr">
-        <is>
-          <t>0:4</t>
         </is>
       </c>
     </row>
@@ -2248,37 +2248,37 @@
       </c>
       <c r="H19" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I19" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="I19" s="21" t="inlineStr">
+      <c r="J19" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J19" s="21" t="inlineStr">
+      <c r="K19" s="21" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="L19" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="K19" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="L19" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
       <c r="M19" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N19" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
-        </is>
-      </c>
-      <c r="N19" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
         </is>
       </c>
     </row>
@@ -2325,32 +2325,32 @@
       </c>
       <c r="I20" s="21" t="inlineStr">
         <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="J20" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="J20" s="21" t="inlineStr">
+      <c r="K20" s="21" t="inlineStr">
         <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="K20" s="21" t="inlineStr">
+      <c r="L20" s="21" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="M20" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="L20" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="M20" s="21" t="inlineStr">
+      <c r="N20" s="21" t="inlineStr">
         <is>
           <t>5:1</t>
-        </is>
-      </c>
-      <c r="N20" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
         </is>
       </c>
     </row>
@@ -2397,32 +2397,32 @@
       </c>
       <c r="I21" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="J21" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="J21" s="21" t="inlineStr">
+      <c r="K21" s="21" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="L21" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K21" s="21" t="inlineStr">
+      <c r="M21" s="21" t="inlineStr">
         <is>
           <t>2:3</t>
         </is>
       </c>
-      <c r="L21" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M21" s="21" t="inlineStr">
+      <c r="N21" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
-        </is>
-      </c>
-      <c r="N21" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
         </is>
       </c>
     </row>
@@ -2464,37 +2464,37 @@
       </c>
       <c r="H22" s="21" t="inlineStr">
         <is>
+          <t>3:2</t>
+        </is>
+      </c>
+      <c r="I22" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="I22" s="21" t="inlineStr">
+      <c r="J22" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="J22" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="K22" s="21" t="inlineStr">
         <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="L22" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="M22" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="L22" s="21" t="inlineStr">
-        <is>
-          <t>3:2</t>
-        </is>
-      </c>
-      <c r="M22" s="21" t="inlineStr">
+      <c r="N22" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
-        </is>
-      </c>
-      <c r="N22" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
         </is>
       </c>
     </row>
@@ -2543,14 +2543,14 @@
       </c>
       <c r="H24" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="I24" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="I24" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="J24" s="21" t="inlineStr">
         <is>
           <t>2:1</t>
@@ -2558,17 +2558,17 @@
       </c>
       <c r="K24" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="L24" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M24" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
-        </is>
-      </c>
-      <c r="L24" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M24" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
         </is>
       </c>
       <c r="N24" s="21" t="inlineStr">
@@ -2620,32 +2620,32 @@
       </c>
       <c r="I25" s="21" t="inlineStr">
         <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="J25" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="J25" s="21" t="inlineStr">
+      <c r="K25" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K25" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="L25" s="21" t="inlineStr">
         <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="M25" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N25" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
-        </is>
-      </c>
-      <c r="M25" s="21" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="N25" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
         </is>
       </c>
     </row>
@@ -2687,37 +2687,37 @@
       </c>
       <c r="H26" s="21" t="inlineStr">
         <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="I26" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I26" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J26" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K26" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K26" s="21" t="inlineStr">
+      <c r="L26" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="M26" s="21" t="inlineStr">
         <is>
           <t>3:3</t>
         </is>
       </c>
-      <c r="L26" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="M26" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N26" s="21" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -2759,37 +2759,37 @@
       </c>
       <c r="H27" s="21" t="inlineStr">
         <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="I27" s="21" t="inlineStr">
+        <is>
           <t>0:0</t>
         </is>
       </c>
-      <c r="I27" s="21" t="inlineStr">
+      <c r="J27" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="J27" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="K27" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="L27" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="M27" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="L27" s="21" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="M27" s="21" t="inlineStr">
+      <c r="N27" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N27" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
         </is>
       </c>
     </row>
@@ -2831,37 +2831,37 @@
       </c>
       <c r="H28" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I28" s="21" t="inlineStr">
+        <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="I28" s="21" t="inlineStr">
+      <c r="J28" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J28" s="21" t="inlineStr">
+      <c r="K28" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="L28" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="K28" s="21" t="inlineStr">
+      <c r="M28" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="L28" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
-      <c r="M28" s="21" t="inlineStr">
+      <c r="N28" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N28" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -2903,37 +2903,37 @@
       </c>
       <c r="H29" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="I29" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="J29" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K29" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L29" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K29" s="21" t="inlineStr">
+      <c r="M29" s="21" t="inlineStr">
         <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="L29" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="M29" s="21" t="inlineStr">
+      <c r="N29" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
-        </is>
-      </c>
-      <c r="N29" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -2982,37 +2982,37 @@
       </c>
       <c r="H31" s="21" t="inlineStr">
         <is>
+          <t>5:0</t>
+        </is>
+      </c>
+      <c r="I31" s="21" t="inlineStr">
+        <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr">
+      <c r="J31" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="J31" s="21" t="inlineStr">
+      <c r="K31" s="21" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="L31" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="K31" s="21" t="inlineStr">
+      <c r="M31" s="21" t="inlineStr">
         <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="L31" s="21" t="inlineStr">
-        <is>
-          <t>5:0</t>
-        </is>
-      </c>
-      <c r="M31" s="21" t="inlineStr">
+      <c r="N31" s="21" t="inlineStr">
         <is>
           <t>7:0</t>
-        </is>
-      </c>
-      <c r="N31" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
         </is>
       </c>
     </row>
@@ -3054,32 +3054,32 @@
       </c>
       <c r="H32" s="21" t="inlineStr">
         <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="I32" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="I32" s="21" t="inlineStr">
+      <c r="J32" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J32" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="K32" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="L32" s="21" t="inlineStr">
         <is>
-          <t>2:3</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="M32" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="N32" s="21" t="inlineStr">
@@ -3126,37 +3126,37 @@
       </c>
       <c r="H33" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>3:2</t>
         </is>
       </c>
       <c r="I33" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="J33" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="K33" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L33" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M33" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="L33" s="21" t="inlineStr">
-        <is>
-          <t>3:2</t>
-        </is>
-      </c>
-      <c r="M33" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="N33" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -3198,7 +3198,7 @@
       </c>
       <c r="H34" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="I34" s="21" t="inlineStr">
@@ -3208,27 +3208,27 @@
       </c>
       <c r="J34" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="K34" s="21" t="inlineStr">
         <is>
+          <t>1:0</t>
+        </is>
+      </c>
+      <c r="L34" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M34" s="21" t="inlineStr">
+        <is>
           <t>3:2</t>
         </is>
       </c>
-      <c r="L34" s="21" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="M34" s="21" t="inlineStr">
+      <c r="N34" s="21" t="inlineStr">
         <is>
           <t>5:0</t>
-        </is>
-      </c>
-      <c r="N34" s="21" t="inlineStr">
-        <is>
-          <t>1:0</t>
         </is>
       </c>
     </row>
@@ -3270,32 +3270,32 @@
       </c>
       <c r="H35" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="I35" s="21" t="inlineStr">
+        <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="I35" s="21" t="inlineStr">
+      <c r="J35" s="21" t="inlineStr">
         <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="J35" s="21" t="inlineStr">
+      <c r="K35" s="21" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="L35" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K35" s="21" t="inlineStr">
+      <c r="M35" s="21" t="inlineStr">
         <is>
           <t>0:0</t>
-        </is>
-      </c>
-      <c r="L35" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M35" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
         </is>
       </c>
       <c r="N35" s="21" t="inlineStr">
@@ -3342,37 +3342,37 @@
       </c>
       <c r="H36" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="I36" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="I36" s="21" t="inlineStr">
+      <c r="J36" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J36" s="21" t="inlineStr">
+      <c r="K36" s="21" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="L36" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K36" s="21" t="inlineStr">
+      <c r="M36" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="L36" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M36" s="21" t="inlineStr">
+      <c r="N36" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N36" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
         </is>
       </c>
     </row>
@@ -3421,37 +3421,37 @@
       </c>
       <c r="H38" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I38" s="21" t="inlineStr">
+        <is>
           <t>0:0</t>
         </is>
       </c>
-      <c r="I38" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="J38" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="K38" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="L38" s="21" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="M38" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="N38" s="21" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -3493,27 +3493,27 @@
       </c>
       <c r="H39" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:0</t>
         </is>
       </c>
       <c r="I39" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="J39" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J39" s="21" t="inlineStr">
+      <c r="K39" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L39" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="K39" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
-      <c r="L39" s="21" t="inlineStr">
-        <is>
-          <t>1:0</t>
         </is>
       </c>
       <c r="M39" s="21" t="inlineStr">
@@ -3570,7 +3570,7 @@
       </c>
       <c r="I40" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="J40" s="21" t="inlineStr">
@@ -3580,22 +3580,22 @@
       </c>
       <c r="K40" s="21" t="inlineStr">
         <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="L40" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="M40" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="L40" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="M40" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N40" s="21" t="inlineStr">
         <is>
-          <t>0:0</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -3637,32 +3637,32 @@
       </c>
       <c r="H41" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="I41" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="I41" s="21" t="inlineStr">
+      <c r="J41" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J41" s="21" t="inlineStr">
+      <c r="K41" s="21" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="L41" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K41" s="21" t="inlineStr">
+      <c r="M41" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="L41" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M41" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
         </is>
       </c>
       <c r="N41" s="21" t="inlineStr">
@@ -3709,32 +3709,32 @@
       </c>
       <c r="H42" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I42" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="I42" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="J42" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="K42" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K42" s="21" t="inlineStr">
+      <c r="L42" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="M42" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
-        </is>
-      </c>
-      <c r="L42" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
-      <c r="M42" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
       <c r="N42" s="21" t="inlineStr">
@@ -3781,37 +3781,37 @@
       </c>
       <c r="H43" s="21" t="inlineStr">
         <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="I43" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="I43" s="21" t="inlineStr">
+      <c r="J43" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J43" s="21" t="inlineStr">
+      <c r="K43" s="21" t="inlineStr">
+        <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="L43" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="K43" s="21" t="inlineStr">
+      <c r="M43" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="L43" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
-        </is>
-      </c>
-      <c r="M43" s="21" t="inlineStr">
+      <c r="N43" s="21" t="inlineStr">
         <is>
           <t>0:1</t>
-        </is>
-      </c>
-      <c r="N43" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
         </is>
       </c>
     </row>
@@ -3860,14 +3860,14 @@
       </c>
       <c r="H45" s="21" t="inlineStr">
         <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="I45" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I45" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="J45" s="21" t="inlineStr">
         <is>
           <t>2:1</t>
@@ -3875,22 +3875,22 @@
       </c>
       <c r="K45" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="L45" s="21" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="M45" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="N45" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
-        </is>
-      </c>
-      <c r="N45" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -3932,32 +3932,32 @@
       </c>
       <c r="H46" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="I46" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I46" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J46" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K46" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K46" s="21" t="inlineStr">
+      <c r="L46" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="M46" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
-        </is>
-      </c>
-      <c r="L46" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="M46" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
       <c r="N46" s="21" t="inlineStr">
@@ -4004,27 +4004,27 @@
       </c>
       <c r="H47" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="I47" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J47" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="J47" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="K47" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>3:0</t>
         </is>
       </c>
       <c r="L47" s="21" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="M47" s="21" t="inlineStr">
@@ -4034,7 +4034,7 @@
       </c>
       <c r="N47" s="21" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -4076,37 +4076,37 @@
       </c>
       <c r="H48" s="21" t="inlineStr">
         <is>
+          <t>2:3</t>
+        </is>
+      </c>
+      <c r="I48" s="21" t="inlineStr">
+        <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="I48" s="21" t="inlineStr">
+      <c r="J48" s="21" t="inlineStr">
         <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="J48" s="21" t="inlineStr">
+      <c r="K48" s="21" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="L48" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K48" s="21" t="inlineStr">
+      <c r="M48" s="21" t="inlineStr">
         <is>
           <t>4:2</t>
         </is>
       </c>
-      <c r="L48" s="21" t="inlineStr">
-        <is>
-          <t>2:3</t>
-        </is>
-      </c>
-      <c r="M48" s="21" t="inlineStr">
+      <c r="N48" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N48" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
         </is>
       </c>
     </row>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="H49" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="I49" s="21" t="inlineStr">
@@ -4158,27 +4158,27 @@
       </c>
       <c r="J49" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="K49" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L49" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="K49" s="21" t="inlineStr">
+      <c r="M49" s="21" t="inlineStr">
         <is>
           <t>3:2</t>
         </is>
       </c>
-      <c r="L49" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="M49" s="21" t="inlineStr">
+      <c r="N49" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
-        </is>
-      </c>
-      <c r="N49" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -4220,32 +4220,32 @@
       </c>
       <c r="H50" s="21" t="inlineStr">
         <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="I50" s="21" t="inlineStr">
+        <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="I50" s="21" t="inlineStr">
+      <c r="J50" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="J50" s="21" t="inlineStr">
+      <c r="K50" s="21" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="L50" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K50" s="21" t="inlineStr">
+      <c r="M50" s="21" t="inlineStr">
         <is>
           <t>1:3</t>
-        </is>
-      </c>
-      <c r="L50" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="M50" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
         </is>
       </c>
       <c r="N50" s="21" t="inlineStr">
@@ -4299,37 +4299,37 @@
       </c>
       <c r="H52" s="21" t="inlineStr">
         <is>
+          <t>7:0</t>
+        </is>
+      </c>
+      <c r="I52" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="I52" s="21" t="inlineStr">
+      <c r="J52" s="21" t="inlineStr">
         <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="J52" s="21" t="inlineStr">
+      <c r="K52" s="21" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="L52" s="21" t="inlineStr">
         <is>
           <t>5:0</t>
         </is>
       </c>
-      <c r="K52" s="21" t="inlineStr">
+      <c r="M52" s="21" t="inlineStr">
         <is>
           <t>5:0</t>
         </is>
       </c>
-      <c r="L52" s="21" t="inlineStr">
-        <is>
-          <t>7:0</t>
-        </is>
-      </c>
-      <c r="M52" s="21" t="inlineStr">
+      <c r="N52" s="21" t="inlineStr">
         <is>
           <t>6:0</t>
-        </is>
-      </c>
-      <c r="N52" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
         </is>
       </c>
     </row>
@@ -4376,32 +4376,32 @@
       </c>
       <c r="I53" s="21" t="inlineStr">
         <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="J53" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="J53" s="21" t="inlineStr">
+      <c r="K53" s="21" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="L53" s="21" t="inlineStr">
         <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="K53" s="21" t="inlineStr">
+      <c r="M53" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="L53" s="21" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="M53" s="21" t="inlineStr">
+      <c r="N53" s="21" t="inlineStr">
         <is>
           <t>0:1</t>
-        </is>
-      </c>
-      <c r="N53" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
         </is>
       </c>
     </row>
@@ -4443,37 +4443,37 @@
       </c>
       <c r="H54" s="21" t="inlineStr">
         <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="I54" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="I54" s="21" t="inlineStr">
+      <c r="J54" s="21" t="inlineStr">
         <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="J54" s="21" t="inlineStr">
+      <c r="K54" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="K54" s="21" t="inlineStr">
+      <c r="L54" s="21" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="M54" s="21" t="inlineStr">
         <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="L54" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
-      <c r="M54" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="N54" s="21" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -4515,14 +4515,14 @@
       </c>
       <c r="H55" s="21" t="inlineStr">
         <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="I55" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I55" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J55" s="21" t="inlineStr">
         <is>
           <t>2:0</t>
@@ -4530,22 +4530,22 @@
       </c>
       <c r="K55" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="L55" s="21" t="inlineStr">
         <is>
-          <t>4:0</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="M55" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N55" s="21" t="inlineStr">
+        <is>
           <t>5:0</t>
-        </is>
-      </c>
-      <c r="N55" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
         </is>
       </c>
     </row>
@@ -4592,32 +4592,32 @@
       </c>
       <c r="I56" s="21" t="inlineStr">
         <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="J56" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="J56" s="21" t="inlineStr">
+      <c r="K56" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L56" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="K56" s="21" t="inlineStr">
+      <c r="M56" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="L56" s="21" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="M56" s="21" t="inlineStr">
+      <c r="N56" s="21" t="inlineStr">
         <is>
           <t>0:4</t>
-        </is>
-      </c>
-      <c r="N56" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -4659,32 +4659,32 @@
       </c>
       <c r="H57" s="21" t="inlineStr">
         <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="I57" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="I57" s="21" t="inlineStr">
+      <c r="J57" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J57" s="21" t="inlineStr">
+      <c r="K57" s="21" t="inlineStr">
+        <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="L57" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K57" s="21" t="inlineStr">
+      <c r="M57" s="21" t="inlineStr">
         <is>
           <t>1:4</t>
-        </is>
-      </c>
-      <c r="L57" s="21" t="inlineStr">
-        <is>
-          <t>2:4</t>
-        </is>
-      </c>
-      <c r="M57" s="21" t="inlineStr">
-        <is>
-          <t>1:2</t>
         </is>
       </c>
       <c r="N57" s="21" t="inlineStr">
@@ -4738,37 +4738,37 @@
       </c>
       <c r="H59" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:2</t>
         </is>
       </c>
       <c r="I59" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J59" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="J59" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="K59" s="21" t="inlineStr">
         <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="L59" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="M59" s="21" t="inlineStr">
+        <is>
           <t>4:1</t>
         </is>
       </c>
-      <c r="L59" s="21" t="inlineStr">
-        <is>
-          <t>4:2</t>
-        </is>
-      </c>
-      <c r="M59" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N59" s="21" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -4810,32 +4810,32 @@
       </c>
       <c r="H60" s="21" t="inlineStr">
         <is>
+          <t>0:1</t>
+        </is>
+      </c>
+      <c r="I60" s="21" t="inlineStr">
+        <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="I60" s="21" t="inlineStr">
+      <c r="J60" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="J60" s="21" t="inlineStr">
+      <c r="K60" s="21" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="L60" s="21" t="inlineStr">
         <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="K60" s="21" t="inlineStr">
+      <c r="M60" s="21" t="inlineStr">
         <is>
           <t>1:4</t>
-        </is>
-      </c>
-      <c r="L60" s="21" t="inlineStr">
-        <is>
-          <t>0:1</t>
-        </is>
-      </c>
-      <c r="M60" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
         </is>
       </c>
       <c r="N60" s="21" t="inlineStr">
@@ -4882,37 +4882,37 @@
       </c>
       <c r="H61" s="21" t="inlineStr">
         <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="I61" s="21" t="inlineStr">
+        <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="I61" s="21" t="inlineStr">
+      <c r="J61" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="J61" s="21" t="inlineStr">
+      <c r="K61" s="21" t="inlineStr">
+        <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="L61" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="K61" s="21" t="inlineStr">
+      <c r="M61" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="L61" s="21" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="M61" s="21" t="inlineStr">
+      <c r="N61" s="21" t="inlineStr">
         <is>
           <t>3:1</t>
-        </is>
-      </c>
-      <c r="N61" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
         </is>
       </c>
     </row>
@@ -4954,7 +4954,7 @@
       </c>
       <c r="H62" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="I62" s="21" t="inlineStr">
@@ -4964,27 +4964,27 @@
       </c>
       <c r="J62" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="K62" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K62" s="21" t="inlineStr">
+      <c r="L62" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="M62" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="L62" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
-      <c r="M62" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N62" s="21" t="inlineStr">
         <is>
-          <t>1:1</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -5026,37 +5026,37 @@
       </c>
       <c r="H63" s="21" t="inlineStr">
         <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="I63" s="21" t="inlineStr">
+        <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="I63" s="21" t="inlineStr">
+      <c r="J63" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J63" s="21" t="inlineStr">
+      <c r="K63" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K63" s="21" t="inlineStr">
+      <c r="L63" s="21" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="M63" s="21" t="inlineStr">
         <is>
           <t>1:4</t>
         </is>
       </c>
-      <c r="L63" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="M63" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="N63" s="21" t="inlineStr">
         <is>
-          <t>0:2</t>
+          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -5098,37 +5098,37 @@
       </c>
       <c r="H64" s="21" t="inlineStr">
         <is>
+          <t>5:2</t>
+        </is>
+      </c>
+      <c r="I64" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="I64" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J64" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="K64" s="21" t="inlineStr">
         <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="L64" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M64" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="L64" s="21" t="inlineStr">
-        <is>
-          <t>5:2</t>
-        </is>
-      </c>
-      <c r="M64" s="21" t="inlineStr">
+      <c r="N64" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="N64" s="21" t="inlineStr">
-        <is>
-          <t>0:0</t>
         </is>
       </c>
     </row>
@@ -5177,37 +5177,37 @@
       </c>
       <c r="H66" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="I66" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="J66" s="21" t="inlineStr">
+        <is>
           <t>4:1</t>
         </is>
       </c>
-      <c r="J66" s="21" t="inlineStr">
+      <c r="K66" s="21" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="L66" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="K66" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="L66" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
-        </is>
-      </c>
       <c r="M66" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="N66" s="21" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -5249,37 +5249,37 @@
       </c>
       <c r="H67" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="I67" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J67" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="J67" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="K67" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:0</t>
         </is>
       </c>
       <c r="L67" s="21" t="inlineStr">
         <is>
-          <t>4:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="M67" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N67" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
-        </is>
-      </c>
-      <c r="N67" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
         </is>
       </c>
     </row>
@@ -5321,19 +5321,19 @@
       </c>
       <c r="H68" s="21" t="inlineStr">
         <is>
+          <t>3:2</t>
+        </is>
+      </c>
+      <c r="I68" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I68" s="21" t="inlineStr">
+      <c r="J68" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J68" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="K68" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
@@ -5341,17 +5341,17 @@
       </c>
       <c r="L68" s="21" t="inlineStr">
         <is>
-          <t>3:2</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="M68" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:2</t>
         </is>
       </c>
       <c r="N68" s="21" t="inlineStr">
         <is>
-          <t>2:2</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -5403,27 +5403,27 @@
       </c>
       <c r="J69" s="21" t="inlineStr">
         <is>
+          <t>1:2</t>
+        </is>
+      </c>
+      <c r="K69" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L69" s="21" t="inlineStr">
+        <is>
           <t>0:1</t>
         </is>
       </c>
-      <c r="K69" s="21" t="inlineStr">
+      <c r="M69" s="21" t="inlineStr">
         <is>
           <t>0:0</t>
         </is>
       </c>
-      <c r="L69" s="21" t="inlineStr">
-        <is>
-          <t>1:2</t>
-        </is>
-      </c>
-      <c r="M69" s="21" t="inlineStr">
+      <c r="N69" s="21" t="inlineStr">
         <is>
           <t>0:1</t>
-        </is>
-      </c>
-      <c r="N69" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -5465,27 +5465,27 @@
       </c>
       <c r="H70" s="21" t="inlineStr">
         <is>
+          <t>2:4</t>
+        </is>
+      </c>
+      <c r="I70" s="21" t="inlineStr">
+        <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="I70" s="21" t="inlineStr">
+      <c r="J70" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J70" s="21" t="inlineStr">
+      <c r="K70" s="21" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="L70" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
-        </is>
-      </c>
-      <c r="K70" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
-        </is>
-      </c>
-      <c r="L70" s="21" t="inlineStr">
-        <is>
-          <t>2:4</t>
         </is>
       </c>
       <c r="M70" s="21" t="inlineStr">
@@ -5537,37 +5537,37 @@
       </c>
       <c r="H71" s="21" t="inlineStr">
         <is>
+          <t>0:5</t>
+        </is>
+      </c>
+      <c r="I71" s="21" t="inlineStr">
+        <is>
           <t>1:3</t>
         </is>
       </c>
-      <c r="I71" s="21" t="inlineStr">
+      <c r="J71" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="J71" s="21" t="inlineStr">
+      <c r="K71" s="21" t="inlineStr">
+        <is>
+          <t>0:4</t>
+        </is>
+      </c>
+      <c r="L71" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="K71" s="21" t="inlineStr">
+      <c r="M71" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="L71" s="21" t="inlineStr">
-        <is>
-          <t>0:5</t>
-        </is>
-      </c>
-      <c r="M71" s="21" t="inlineStr">
+      <c r="N71" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
-        </is>
-      </c>
-      <c r="N71" s="21" t="inlineStr">
-        <is>
-          <t>0:4</t>
         </is>
       </c>
     </row>
@@ -5616,37 +5616,37 @@
       </c>
       <c r="H73" s="21" t="inlineStr">
         <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="I73" s="21" t="inlineStr">
+        <is>
           <t>1:0</t>
         </is>
       </c>
-      <c r="I73" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="J73" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="K73" s="21" t="inlineStr">
+        <is>
+          <t>3:1</t>
+        </is>
+      </c>
+      <c r="L73" s="21" t="inlineStr">
+        <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="K73" s="21" t="inlineStr">
+      <c r="M73" s="21" t="inlineStr">
         <is>
           <t>5:1</t>
         </is>
       </c>
-      <c r="L73" s="21" t="inlineStr">
-        <is>
-          <t>3:0</t>
-        </is>
-      </c>
-      <c r="M73" s="21" t="inlineStr">
+      <c r="N73" s="21" t="inlineStr">
         <is>
           <t>4:0</t>
-        </is>
-      </c>
-      <c r="N73" s="21" t="inlineStr">
-        <is>
-          <t>3:1</t>
         </is>
       </c>
     </row>
@@ -5693,32 +5693,32 @@
       </c>
       <c r="I74" s="21" t="inlineStr">
         <is>
+          <t>1:3</t>
+        </is>
+      </c>
+      <c r="J74" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J74" s="21" t="inlineStr">
+      <c r="K74" s="21" t="inlineStr">
+        <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="L74" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K74" s="21" t="inlineStr">
+      <c r="M74" s="21" t="inlineStr">
         <is>
           <t>2:2</t>
         </is>
       </c>
-      <c r="L74" s="21" t="inlineStr">
-        <is>
-          <t>1:3</t>
-        </is>
-      </c>
-      <c r="M74" s="21" t="inlineStr">
+      <c r="N74" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
-        </is>
-      </c>
-      <c r="N74" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
         </is>
       </c>
     </row>
@@ -5760,37 +5760,37 @@
       </c>
       <c r="H75" s="21" t="inlineStr">
         <is>
+          <t>4:0</t>
+        </is>
+      </c>
+      <c r="I75" s="21" t="inlineStr">
+        <is>
           <t>4:1</t>
         </is>
       </c>
-      <c r="I75" s="21" t="inlineStr">
+      <c r="J75" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="J75" s="21" t="inlineStr">
+      <c r="K75" s="21" t="inlineStr">
+        <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="L75" s="21" t="inlineStr">
         <is>
           <t>5:0</t>
         </is>
       </c>
-      <c r="K75" s="21" t="inlineStr">
+      <c r="M75" s="21" t="inlineStr">
         <is>
           <t>3:0</t>
         </is>
       </c>
-      <c r="L75" s="21" t="inlineStr">
-        <is>
-          <t>4:0</t>
-        </is>
-      </c>
-      <c r="M75" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N75" s="21" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -5832,32 +5832,32 @@
       </c>
       <c r="H76" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>4:1</t>
         </is>
       </c>
       <c r="I76" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="J76" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="J76" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="K76" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="L76" s="21" t="inlineStr">
+        <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="M76" s="21" t="inlineStr">
+        <is>
           <t>2:2</t>
-        </is>
-      </c>
-      <c r="L76" s="21" t="inlineStr">
-        <is>
-          <t>4:1</t>
-        </is>
-      </c>
-      <c r="M76" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
         </is>
       </c>
       <c r="N76" s="21" t="inlineStr">
@@ -5909,32 +5909,32 @@
       </c>
       <c r="I77" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="J77" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="J77" s="21" t="inlineStr">
+      <c r="K77" s="21" t="inlineStr">
+        <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L77" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="K77" s="21" t="inlineStr">
+      <c r="M77" s="21" t="inlineStr">
         <is>
           <t>1:4</t>
         </is>
       </c>
-      <c r="L77" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
-      <c r="M77" s="21" t="inlineStr">
+      <c r="N77" s="21" t="inlineStr">
         <is>
           <t>0:0</t>
-        </is>
-      </c>
-      <c r="N77" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -5976,32 +5976,32 @@
       </c>
       <c r="H78" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>0:0</t>
         </is>
       </c>
       <c r="I78" s="21" t="inlineStr">
         <is>
+          <t>2:0</t>
+        </is>
+      </c>
+      <c r="J78" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="J78" s="21" t="inlineStr">
+      <c r="K78" s="21" t="inlineStr">
+        <is>
+          <t>0:0</t>
+        </is>
+      </c>
+      <c r="L78" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K78" s="21" t="inlineStr">
+      <c r="M78" s="21" t="inlineStr">
         <is>
           <t>3:2</t>
-        </is>
-      </c>
-      <c r="L78" s="21" t="inlineStr">
-        <is>
-          <t>0:0</t>
-        </is>
-      </c>
-      <c r="M78" s="21" t="inlineStr">
-        <is>
-          <t>0:0</t>
         </is>
       </c>
       <c r="N78" s="21" t="inlineStr">
@@ -6055,7 +6055,7 @@
       </c>
       <c r="H80" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>1:1</t>
         </is>
       </c>
       <c r="I80" s="21" t="inlineStr">
@@ -6065,27 +6065,27 @@
       </c>
       <c r="J80" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="K80" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="L80" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M80" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="L80" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
-        </is>
-      </c>
-      <c r="M80" s="21" t="inlineStr">
+      <c r="N80" s="21" t="inlineStr">
         <is>
           <t>1:2</t>
-        </is>
-      </c>
-      <c r="N80" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
         </is>
       </c>
     </row>
@@ -6137,7 +6137,7 @@
       </c>
       <c r="J81" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>3:1</t>
         </is>
       </c>
       <c r="K81" s="21" t="inlineStr">
@@ -6147,17 +6147,17 @@
       </c>
       <c r="L81" s="21" t="inlineStr">
         <is>
-          <t>3:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="M81" s="21" t="inlineStr">
         <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="N81" s="21" t="inlineStr">
+        <is>
           <t>3:0</t>
-        </is>
-      </c>
-      <c r="N81" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
         </is>
       </c>
     </row>
@@ -6199,7 +6199,7 @@
       </c>
       <c r="H82" s="21" t="inlineStr">
         <is>
-          <t>2:0</t>
+          <t>2:1</t>
         </is>
       </c>
       <c r="I82" s="21" t="inlineStr">
@@ -6209,27 +6209,27 @@
       </c>
       <c r="J82" s="21" t="inlineStr">
         <is>
-          <t>2:1</t>
+          <t>2:0</t>
         </is>
       </c>
       <c r="K82" s="21" t="inlineStr">
         <is>
+          <t>3:0</t>
+        </is>
+      </c>
+      <c r="L82" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M82" s="21" t="inlineStr">
+        <is>
           <t>4:0</t>
         </is>
       </c>
-      <c r="L82" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
-      <c r="M82" s="21" t="inlineStr">
-        <is>
-          <t>2:0</t>
-        </is>
-      </c>
       <c r="N82" s="21" t="inlineStr">
         <is>
-          <t>3:0</t>
+          <t>2:0</t>
         </is>
       </c>
     </row>
@@ -6271,32 +6271,32 @@
       </c>
       <c r="H83" s="21" t="inlineStr">
         <is>
+          <t>1:4</t>
+        </is>
+      </c>
+      <c r="I83" s="21" t="inlineStr">
+        <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="I83" s="21" t="inlineStr">
+      <c r="J83" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="J83" s="21" t="inlineStr">
+      <c r="K83" s="21" t="inlineStr">
+        <is>
+          <t>0:2</t>
+        </is>
+      </c>
+      <c r="L83" s="21" t="inlineStr">
         <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="K83" s="21" t="inlineStr">
+      <c r="M83" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
-        </is>
-      </c>
-      <c r="L83" s="21" t="inlineStr">
-        <is>
-          <t>1:4</t>
-        </is>
-      </c>
-      <c r="M83" s="21" t="inlineStr">
-        <is>
-          <t>0:2</t>
         </is>
       </c>
       <c r="N83" s="21" t="inlineStr">
@@ -6343,32 +6343,32 @@
       </c>
       <c r="H84" s="21" t="inlineStr">
         <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="I84" s="21" t="inlineStr">
+        <is>
           <t>1:2</t>
         </is>
       </c>
-      <c r="I84" s="21" t="inlineStr">
+      <c r="J84" s="21" t="inlineStr">
         <is>
           <t>0:3</t>
         </is>
       </c>
-      <c r="J84" s="21" t="inlineStr">
+      <c r="K84" s="21" t="inlineStr">
+        <is>
+          <t>0:3</t>
+        </is>
+      </c>
+      <c r="L84" s="21" t="inlineStr">
         <is>
           <t>0:2</t>
         </is>
       </c>
-      <c r="K84" s="21" t="inlineStr">
+      <c r="M84" s="21" t="inlineStr">
         <is>
           <t>1:4</t>
-        </is>
-      </c>
-      <c r="L84" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
-        </is>
-      </c>
-      <c r="M84" s="21" t="inlineStr">
-        <is>
-          <t>0:3</t>
         </is>
       </c>
       <c r="N84" s="21" t="inlineStr">
@@ -6415,14 +6415,14 @@
       </c>
       <c r="H85" s="21" t="inlineStr">
         <is>
+          <t>2:2</t>
+        </is>
+      </c>
+      <c r="I85" s="21" t="inlineStr">
+        <is>
           <t>1:1</t>
         </is>
       </c>
-      <c r="I85" s="21" t="inlineStr">
-        <is>
-          <t>2:1</t>
-        </is>
-      </c>
       <c r="J85" s="21" t="inlineStr">
         <is>
           <t>2:1</t>
@@ -6430,22 +6430,22 @@
       </c>
       <c r="K85" s="21" t="inlineStr">
         <is>
+          <t>1:1</t>
+        </is>
+      </c>
+      <c r="L85" s="21" t="inlineStr">
+        <is>
+          <t>2:1</t>
+        </is>
+      </c>
+      <c r="M85" s="21" t="inlineStr">
+        <is>
           <t>3:1</t>
         </is>
       </c>
-      <c r="L85" s="21" t="inlineStr">
-        <is>
-          <t>2:2</t>
-        </is>
-      </c>
-      <c r="M85" s="21" t="inlineStr">
+      <c r="N85" s="21" t="inlineStr">
         <is>
           <t>1:0</t>
-        </is>
-      </c>
-      <c r="N85" s="21" t="inlineStr">
-        <is>
-          <t>1:1</t>
         </is>
       </c>
     </row>
@@ -6531,37 +6531,37 @@
       </c>
       <c r="H1" s="13" t="inlineStr">
         <is>
+          <t>Christian Sandritter</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
           <t>Egon Hejda</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Friedbert Mechler</t>
         </is>
       </c>
-      <c r="J1" s="13" t="inlineStr">
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>Rony Burkart</t>
+        </is>
+      </c>
+      <c r="L1" s="13" t="inlineStr">
         <is>
           <t>Stefan Seiler</t>
         </is>
       </c>
-      <c r="K1" s="13" t="inlineStr">
+      <c r="M1" s="13" t="inlineStr">
         <is>
           <t>Heiko Baust</t>
         </is>
       </c>
-      <c r="L1" s="13" t="inlineStr">
-        <is>
-          <t>Christian Sandritter</t>
-        </is>
-      </c>
-      <c r="M1" s="13" t="inlineStr">
+      <c r="N1" s="13" t="inlineStr">
         <is>
           <t>Markus Bruckner</t>
-        </is>
-      </c>
-      <c r="N1" s="13" t="inlineStr">
-        <is>
-          <t>Rony Burkart</t>
         </is>
       </c>
     </row>
@@ -6615,32 +6615,32 @@
       </c>
       <c r="I3" s="21" t="inlineStr">
         <is>
+          <t>Südkorea</t>
+        </is>
+      </c>
+      <c r="J3" s="21" t="inlineStr">
+        <is>
           <t>Bosnien-Herzegowina</t>
         </is>
       </c>
-      <c r="J3" s="21" t="inlineStr">
+      <c r="K3" s="21" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+      <c r="L3" s="21" t="inlineStr">
         <is>
           <t>Kanada</t>
         </is>
       </c>
-      <c r="K3" s="21" t="inlineStr">
+      <c r="M3" s="21" t="inlineStr">
         <is>
           <t>Mexiko</t>
         </is>
       </c>
-      <c r="L3" s="21" t="inlineStr">
-        <is>
-          <t>Südkorea</t>
-        </is>
-      </c>
-      <c r="M3" s="21" t="inlineStr">
+      <c r="N3" s="21" t="inlineStr">
         <is>
           <t>Tschechien</t>
-        </is>
-      </c>
-      <c r="N3" s="21" t="inlineStr">
-        <is>
-          <t>Mexiko</t>
         </is>
       </c>
     </row>
@@ -6841,22 +6841,22 @@
       </c>
       <c r="K6" s="21" t="inlineStr">
         <is>
+          <t>Japan</t>
+        </is>
+      </c>
+      <c r="L6" s="21" t="inlineStr">
+        <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="L6" s="21" t="inlineStr">
+      <c r="M6" s="21" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="M6" s="21" t="inlineStr">
+      <c r="N6" s="21" t="inlineStr">
         <is>
           <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="N6" s="21" t="inlineStr">
-        <is>
-          <t>Japan</t>
         </is>
       </c>
     </row>
@@ -6908,27 +6908,27 @@
       </c>
       <c r="J7" s="21" t="inlineStr">
         <is>
+          <t>Norwegen</t>
+        </is>
+      </c>
+      <c r="K7" s="21" t="inlineStr">
+        <is>
           <t>Elfenbeinküste</t>
         </is>
       </c>
-      <c r="K7" s="21" t="inlineStr">
+      <c r="L7" s="21" t="inlineStr">
+        <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+      <c r="M7" s="21" t="inlineStr">
         <is>
           <t>Norwegen</t>
         </is>
       </c>
-      <c r="L7" s="21" t="inlineStr">
-        <is>
-          <t>Norwegen</t>
-        </is>
-      </c>
-      <c r="M7" s="21" t="inlineStr">
+      <c r="N7" s="21" t="inlineStr">
         <is>
           <t>Frankreich</t>
-        </is>
-      </c>
-      <c r="N7" s="21" t="inlineStr">
-        <is>
-          <t>Elfenbeinküste</t>
         </is>
       </c>
     </row>
@@ -6995,12 +6995,12 @@
       </c>
       <c r="M8" s="21" t="inlineStr">
         <is>
+          <t>Frankreich</t>
+        </is>
+      </c>
+      <c r="N8" s="21" t="inlineStr">
+        <is>
           <t>Norwegen</t>
-        </is>
-      </c>
-      <c r="N8" s="21" t="inlineStr">
-        <is>
-          <t>Frankreich</t>
         </is>
       </c>
     </row>
@@ -7067,12 +7067,12 @@
       </c>
       <c r="M9" s="21" t="inlineStr">
         <is>
+          <t>Tschechien</t>
+        </is>
+      </c>
+      <c r="N9" s="21" t="inlineStr">
+        <is>
           <t>Mexiko</t>
-        </is>
-      </c>
-      <c r="N9" s="21" t="inlineStr">
-        <is>
-          <t>Tschechien</t>
         </is>
       </c>
     </row>
@@ -7139,12 +7139,12 @@
       </c>
       <c r="M10" s="21" t="inlineStr">
         <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="N10" s="21" t="inlineStr">
+        <is>
           <t>Kroatien</t>
-        </is>
-      </c>
-      <c r="N10" s="21" t="inlineStr">
-        <is>
-          <t>England</t>
         </is>
       </c>
     </row>
@@ -7258,37 +7258,37 @@
       </c>
       <c r="H12" s="21" t="inlineStr">
         <is>
+          <t>Elfenbeinküste</t>
+        </is>
+      </c>
+      <c r="I12" s="21" t="inlineStr">
+        <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="I12" s="21" t="inlineStr">
+      <c r="J12" s="21" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="J12" s="21" t="inlineStr">
+      <c r="K12" s="21" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
-      <c r="K12" s="21" t="inlineStr">
+      <c r="L12" s="21" t="inlineStr">
+        <is>
+          <t>Türkei</t>
+        </is>
+      </c>
+      <c r="M12" s="21" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="L12" s="21" t="inlineStr">
-        <is>
-          <t>Elfenbeinküste</t>
-        </is>
-      </c>
-      <c r="M12" s="21" t="inlineStr">
+      <c r="N12" s="21" t="inlineStr">
         <is>
           <t>USA</t>
-        </is>
-      </c>
-      <c r="N12" s="21" t="inlineStr">
-        <is>
-          <t>Türkei</t>
         </is>
       </c>
     </row>
@@ -7402,37 +7402,37 @@
       </c>
       <c r="H14" s="21" t="inlineStr">
         <is>
+          <t>Kroatien</t>
+        </is>
+      </c>
+      <c r="I14" s="21" t="inlineStr">
+        <is>
           <t>Kolumbien</t>
         </is>
       </c>
-      <c r="I14" s="21" t="inlineStr">
+      <c r="J14" s="21" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
-      <c r="J14" s="21" t="inlineStr">
+      <c r="K14" s="21" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
-      <c r="K14" s="21" t="inlineStr">
+      <c r="L14" s="21" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
-      <c r="L14" s="21" t="inlineStr">
+      <c r="M14" s="21" t="inlineStr">
         <is>
           <t>Kroatien</t>
         </is>
       </c>
-      <c r="M14" s="21" t="inlineStr">
+      <c r="N14" s="21" t="inlineStr">
         <is>
           <t>England</t>
-        </is>
-      </c>
-      <c r="N14" s="21" t="inlineStr">
-        <is>
-          <t>Kroatien</t>
         </is>
       </c>
     </row>
@@ -7546,37 +7546,37 @@
       </c>
       <c r="H16" s="21" t="inlineStr">
         <is>
+          <t>USA</t>
+        </is>
+      </c>
+      <c r="I16" s="21" t="inlineStr">
+        <is>
           <t>Ägypten</t>
         </is>
       </c>
-      <c r="I16" s="21" t="inlineStr">
+      <c r="J16" s="21" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
-      <c r="J16" s="21" t="inlineStr">
+      <c r="K16" s="21" t="inlineStr">
+        <is>
+          <t>Paraguay</t>
+        </is>
+      </c>
+      <c r="L16" s="21" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="K16" s="21" t="inlineStr">
+      <c r="M16" s="21" t="inlineStr">
         <is>
           <t>Neuseeland</t>
         </is>
       </c>
-      <c r="L16" s="21" t="inlineStr">
-        <is>
-          <t>USA</t>
-        </is>
-      </c>
-      <c r="M16" s="21" t="inlineStr">
+      <c r="N16" s="21" t="inlineStr">
         <is>
           <t>Türkei</t>
-        </is>
-      </c>
-      <c r="N16" s="21" t="inlineStr">
-        <is>
-          <t>Paraguay</t>
         </is>
       </c>
     </row>
@@ -7769,37 +7769,37 @@
       </c>
       <c r="H20" s="21" t="inlineStr">
         <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I20" s="21" t="inlineStr">
+        <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="I20" s="21" t="inlineStr">
+      <c r="J20" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="J20" s="21" t="inlineStr">
+      <c r="K20" s="21" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="L20" s="21" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="K20" s="21" t="inlineStr">
+      <c r="M20" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="L20" s="21" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="M20" s="21" t="inlineStr">
+      <c r="N20" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
-        </is>
-      </c>
-      <c r="N20" s="21" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
         </is>
       </c>
     </row>
@@ -7841,37 +7841,37 @@
       </c>
       <c r="H21" s="21" t="inlineStr">
         <is>
+          <t>Niederlande</t>
+        </is>
+      </c>
+      <c r="I21" s="21" t="inlineStr">
+        <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="I21" s="21" t="inlineStr">
+      <c r="J21" s="21" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="J21" s="21" t="inlineStr">
+      <c r="K21" s="21" t="inlineStr">
+        <is>
+          <t>Mexiko</t>
+        </is>
+      </c>
+      <c r="L21" s="21" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="K21" s="21" t="inlineStr">
+      <c r="M21" s="21" t="inlineStr">
         <is>
           <t>Niederlande</t>
         </is>
       </c>
-      <c r="L21" s="21" t="inlineStr">
-        <is>
-          <t>Niederlande</t>
-        </is>
-      </c>
-      <c r="M21" s="21" t="inlineStr">
+      <c r="N21" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="N21" s="21" t="inlineStr">
-        <is>
-          <t>Mexiko</t>
         </is>
       </c>
     </row>
@@ -7913,37 +7913,37 @@
       </c>
       <c r="H22" s="21" t="inlineStr">
         <is>
+          <t>Norwegen</t>
+        </is>
+      </c>
+      <c r="I22" s="21" t="inlineStr">
+        <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="I22" s="21" t="inlineStr">
+      <c r="J22" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="J22" s="21" t="inlineStr">
+      <c r="K22" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="K22" s="21" t="inlineStr">
+      <c r="L22" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="L22" s="21" t="inlineStr">
+      <c r="M22" s="21" t="inlineStr">
+        <is>
+          <t>Brasilien</t>
+        </is>
+      </c>
+      <c r="N22" s="21" t="inlineStr">
         <is>
           <t>Norwegen</t>
-        </is>
-      </c>
-      <c r="M22" s="21" t="inlineStr">
-        <is>
-          <t>Norwegen</t>
-        </is>
-      </c>
-      <c r="N22" s="21" t="inlineStr">
-        <is>
-          <t>Brasilien</t>
         </is>
       </c>
     </row>
@@ -8010,12 +8010,12 @@
       </c>
       <c r="M23" s="21" t="inlineStr">
         <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="N23" s="21" t="inlineStr">
+        <is>
           <t>Mexiko</t>
-        </is>
-      </c>
-      <c r="N23" s="21" t="inlineStr">
-        <is>
-          <t>England</t>
         </is>
       </c>
     </row>
@@ -8057,37 +8057,37 @@
       </c>
       <c r="H24" s="21" t="inlineStr">
         <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I24" s="21" t="inlineStr">
+        <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="I24" s="21" t="inlineStr">
+      <c r="J24" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="J24" s="21" t="inlineStr">
+      <c r="K24" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="K24" s="21" t="inlineStr">
+      <c r="L24" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="L24" s="21" t="inlineStr">
+      <c r="M24" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="M24" s="21" t="inlineStr">
+      <c r="N24" s="21" t="inlineStr">
         <is>
           <t>Belgien</t>
-        </is>
-      </c>
-      <c r="N24" s="21" t="inlineStr">
-        <is>
-          <t>Spanien</t>
         </is>
       </c>
     </row>
@@ -8129,37 +8129,37 @@
       </c>
       <c r="H25" s="21" t="inlineStr">
         <is>
+          <t>Belgien</t>
+        </is>
+      </c>
+      <c r="I25" s="21" t="inlineStr">
+        <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="I25" s="21" t="inlineStr">
+      <c r="J25" s="21" t="inlineStr">
         <is>
           <t>Belgien</t>
         </is>
       </c>
-      <c r="J25" s="21" t="inlineStr">
+      <c r="K25" s="21" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
-      <c r="K25" s="21" t="inlineStr">
+      <c r="L25" s="21" t="inlineStr">
+        <is>
+          <t>Türkei</t>
+        </is>
+      </c>
+      <c r="M25" s="21" t="inlineStr">
         <is>
           <t>USA</t>
         </is>
       </c>
-      <c r="L25" s="21" t="inlineStr">
-        <is>
-          <t>Belgien</t>
-        </is>
-      </c>
-      <c r="M25" s="21" t="inlineStr">
+      <c r="N25" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
-        </is>
-      </c>
-      <c r="N25" s="21" t="inlineStr">
-        <is>
-          <t>Türkei</t>
         </is>
       </c>
     </row>
@@ -8201,37 +8201,37 @@
       </c>
       <c r="H26" s="21" t="inlineStr">
         <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+      <c r="I26" s="21" t="inlineStr">
+        <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="I26" s="21" t="inlineStr">
+      <c r="J26" s="21" t="inlineStr">
         <is>
           <t>Türkei</t>
         </is>
       </c>
-      <c r="J26" s="21" t="inlineStr">
+      <c r="K26" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="K26" s="21" t="inlineStr">
+      <c r="L26" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="L26" s="21" t="inlineStr">
+      <c r="M26" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="M26" s="21" t="inlineStr">
+      <c r="N26" s="21" t="inlineStr">
         <is>
           <t>Schweiz</t>
-        </is>
-      </c>
-      <c r="N26" s="21" t="inlineStr">
-        <is>
-          <t>Argentinien</t>
         </is>
       </c>
     </row>
@@ -8278,32 +8278,32 @@
       </c>
       <c r="I27" s="21" t="inlineStr">
         <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="J27" s="21" t="inlineStr">
+        <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="J27" s="21" t="inlineStr">
+      <c r="K27" s="21" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="K27" s="21" t="inlineStr">
+      <c r="L27" s="21" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="L27" s="21" t="inlineStr">
+      <c r="M27" s="21" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="M27" s="21" t="inlineStr">
+      <c r="N27" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="N27" s="21" t="inlineStr">
-        <is>
-          <t>Portugal</t>
         </is>
       </c>
     </row>
@@ -8362,27 +8362,27 @@
       </c>
       <c r="J29" s="21" t="inlineStr">
         <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="K29" s="21" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="L29" s="21" t="inlineStr">
+        <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="K29" s="21" t="inlineStr">
+      <c r="M29" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="L29" s="21" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
-        </is>
-      </c>
-      <c r="M29" s="21" t="inlineStr">
+      <c r="N29" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
-        </is>
-      </c>
-      <c r="N29" s="21" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
         </is>
       </c>
     </row>
@@ -8424,37 +8424,37 @@
       </c>
       <c r="H30" s="21" t="inlineStr">
         <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I30" s="21" t="inlineStr">
+        <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="I30" s="21" t="inlineStr">
+      <c r="J30" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="J30" s="21" t="inlineStr">
+      <c r="K30" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="K30" s="21" t="inlineStr">
+      <c r="L30" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="L30" s="21" t="inlineStr">
+      <c r="M30" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="M30" s="21" t="inlineStr">
+      <c r="N30" s="21" t="inlineStr">
         <is>
           <t>Norwegen</t>
-        </is>
-      </c>
-      <c r="N30" s="21" t="inlineStr">
-        <is>
-          <t>Spanien</t>
         </is>
       </c>
     </row>
@@ -8496,37 +8496,37 @@
       </c>
       <c r="H31" s="21" t="inlineStr">
         <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="I31" s="21" t="inlineStr">
+        <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="I31" s="21" t="inlineStr">
+      <c r="J31" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="J31" s="21" t="inlineStr">
+      <c r="K31" s="21" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="L31" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="K31" s="21" t="inlineStr">
+      <c r="M31" s="21" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="L31" s="21" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="M31" s="21" t="inlineStr">
+      <c r="N31" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
-        </is>
-      </c>
-      <c r="N31" s="21" t="inlineStr">
-        <is>
-          <t>England</t>
         </is>
       </c>
     </row>
@@ -8568,37 +8568,37 @@
       </c>
       <c r="H32" s="21" t="inlineStr">
         <is>
+          <t>Argentinien</t>
+        </is>
+      </c>
+      <c r="I32" s="21" t="inlineStr">
+        <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="I32" s="21" t="inlineStr">
+      <c r="J32" s="21" t="inlineStr">
         <is>
           <t>Schweiz</t>
         </is>
       </c>
-      <c r="J32" s="21" t="inlineStr">
+      <c r="K32" s="21" t="inlineStr">
+        <is>
+          <t>Portugal</t>
+        </is>
+      </c>
+      <c r="L32" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="K32" s="21" t="inlineStr">
+      <c r="M32" s="21" t="inlineStr">
         <is>
           <t>Portugal</t>
         </is>
       </c>
-      <c r="L32" s="21" t="inlineStr">
+      <c r="N32" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="M32" s="21" t="inlineStr">
-        <is>
-          <t>Argentinien</t>
-        </is>
-      </c>
-      <c r="N32" s="21" t="inlineStr">
-        <is>
-          <t>Portugal</t>
         </is>
       </c>
     </row>
@@ -8647,37 +8647,37 @@
       </c>
       <c r="H34" s="21" t="inlineStr">
         <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="I34" s="21" t="inlineStr">
+        <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="I34" s="21" t="inlineStr">
+      <c r="J34" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="J34" s="21" t="inlineStr">
+      <c r="K34" s="21" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="L34" s="21" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="K34" s="21" t="inlineStr">
+      <c r="M34" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="L34" s="21" t="inlineStr">
-        <is>
-          <t>Spanien</t>
-        </is>
-      </c>
-      <c r="M34" s="21" t="inlineStr">
+      <c r="N34" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
-        </is>
-      </c>
-      <c r="N34" s="21" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
         </is>
       </c>
     </row>
@@ -8719,37 +8719,37 @@
       </c>
       <c r="H35" s="21" t="inlineStr">
         <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="I35" s="21" t="inlineStr">
+        <is>
           <t>Spanien</t>
         </is>
       </c>
-      <c r="I35" s="21" t="inlineStr">
+      <c r="J35" s="21" t="inlineStr">
         <is>
           <t>Brasilien</t>
         </is>
       </c>
-      <c r="J35" s="21" t="inlineStr">
+      <c r="K35" s="21" t="inlineStr">
+        <is>
+          <t>England</t>
+        </is>
+      </c>
+      <c r="L35" s="21" t="inlineStr">
         <is>
           <t>Argentinien</t>
         </is>
       </c>
-      <c r="K35" s="21" t="inlineStr">
+      <c r="M35" s="21" t="inlineStr">
         <is>
           <t>England</t>
         </is>
       </c>
-      <c r="L35" s="21" t="inlineStr">
-        <is>
-          <t>England</t>
-        </is>
-      </c>
-      <c r="M35" s="21" t="inlineStr">
+      <c r="N35" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
-        </is>
-      </c>
-      <c r="N35" s="21" t="inlineStr">
-        <is>
-          <t>England</t>
         </is>
       </c>
     </row>
@@ -8803,32 +8803,32 @@
       </c>
       <c r="I37" s="21" t="inlineStr">
         <is>
+          <t>Spanien</t>
+        </is>
+      </c>
+      <c r="J37" s="21" t="inlineStr">
+        <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="J37" s="21" t="inlineStr">
+      <c r="K37" s="21" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="L37" s="21" t="inlineStr">
         <is>
           <t>Frankreich</t>
         </is>
       </c>
-      <c r="K37" s="21" t="inlineStr">
+      <c r="M37" s="21" t="inlineStr">
         <is>
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="L37" s="21" t="inlineStr">
+      <c r="N37" s="21" t="inlineStr">
         <is>
           <t>Spanien</t>
-        </is>
-      </c>
-      <c r="M37" s="21" t="inlineStr">
-        <is>
-          <t>Spanien</t>
-        </is>
-      </c>
-      <c r="N37" s="21" t="inlineStr">
-        <is>
-          <t>Deutschland</t>
         </is>
       </c>
     </row>

</xml_diff>